<commit_message>
updated ACF scorecards, updated surveys, and added links to resources page
</commit_message>
<xml_diff>
--- a/website/assets/files/Agency Questionnaire Data Export 2022.xlsx
+++ b/website/assets/files/Agency Questionnaire Data Export 2022.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffhawley/source/omb-payment-accuracy/website/assets/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pajak_hc\Work Folders\Desktop\Heather's Folders\Data Call\FY2025 Data Call\Website\Datasets\Exports of Questionnaires\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{948AE2A1-4D2F-634A-B521-5C09CE7EB731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EB8AD6D-8076-4EC5-B728-C44C7BE7533B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2490" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2022 Agency Survey Q&amp;A" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2022 Agency Survey Q&amp;A'!$A$3:$AV$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2022 Agency Survey Q&amp;A'!$A$3:$AW$56</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="417">
   <si>
     <t>CFTC</t>
   </si>
@@ -1598,6 +1601,221 @@
     <t>HHS conduct recovery audits in Medicare, and states conduct recovery audits in Medicaid.  CMS collects improper payments identified via recovery audits by the issuance of a "Demand" letter.  The amount owed could be collected via an offset from future  payments or a provider could submit a refund to the Medicare Administrative Contractor.  In addition, debts can also be referred to the Department of Treasury for collection.</t>
   </si>
   <si>
+    <t>OSC monitors various aspects of its financial activities throughout the year, including spot reviews of the agency's transit subsidy usage, analysis of expected payroll and benefits against the actual payroll and benefits, etc., and addresses any instances where overpayments are identified.</t>
+  </si>
+  <si>
+    <t>Bills of collection, offset of future payments, Treasury CRS</t>
+  </si>
+  <si>
+    <t>Recapture audits were performed internally instead of by a external contractor.</t>
+  </si>
+  <si>
+    <t>Invoices processed through the Invoice Processing Platform (IPP) are subject to a monthly post payment audit of 10% of the total paid IPP invoices for that month.  Invoices not processed through the Invoice Processing Platform (IPP) in excess of $2,500.00 are subject to secondary review before being paid.  Invoices under $2,500.00 are subject to review through statistical sampling procedures.  Travel vouchers processed through the Concur Government Edition (CGE) travel system are subject to a post payment audit based on a random sample of all reimbursements under $2,500.   All payments of $2,500.00 and higher are excluded from the population. These payments require a 100% post payment audit review. Relocation vouchers processed through the MoveLINQ system are subject to 100% pre-payment audit and review.   For payment customers, once the vouchers have been pre-audited and approved for payment, they are interfaced to the Oracle the financial system through which they are paid.   
+The DNP portal implementation has provided a way for our procurement and payable offices to review vendor files prior to disbursement.  It has also given us an opportunity to review the monthly payment file results to identify any improper payments made to a vendor in the DNP portal.</t>
+  </si>
+  <si>
+    <t>VA has established recovery audits in a manner that maximizes efficiency; therefore, many programs' payments are audited for overpayments that can be recovered using the same processes and procedures. At VA, these audits are performed in five major areas: Veterans Health Administration for several unique programs providing health care, Veterans Benefits Administration for benefit programs where the Financial Services Center in Austin, Texas does not process their payments, the Financial Services Center which provides recovery audits for all payments it processes which includes Veterans Health Administration payments, some Veterans Benefits Administration payments, National Cemetery Administration payments, and VA's Staff Offices (for example, Office of Information Technology, Office of Management, and the Office of Human Resources &amp; Administration/Operations, Security &amp; Preparedness), as well as specific recovery audits performed by the Office of Inspector General's additional shared service providers for payroll and Supply Fund payments in the Office of Revolving Fund. These are discussed in more detail below.
+Veterans Health Administration
+Veterans Health Administration is operationalizing a recovery audit contract which will audit claims from FY 2018 through FY 2023 for Civilian Health and Medical Program of the Department of Veterans Affairs, Veterans Health Administration Spina Bifida Health Care, and VA Community Care programs. The review includes inpatient claims paid under the following authorities: 38 U.S.C. § 1703 (authorized care); 38 U.S.C. § 1728 (service connected unauthorized care); and 38 U.S.C. § 1725 (non-service connected emergency care) and will test to ensure the care rendered is in compliance with the authorization/referral; was reimbursed based on the appropriate methodology; and that the medical records support the diagnostic related group billed for the services.
+Veterans Benefits Administration
+Veterans Benefits Administration uses a combination of quality reviews and payment reviews to identify possible duplicates and overpayments. The majority of Veterans Benefits Administration programs perform quality reviews on randomly selected cases that ensure eligibility determinations, proper case processing, and payment accuracy. For all other programs, Veterans Benefits Administration performs payment reviews to identify potential duplicate payments and other potential improper payments. Veterans Benefits Administration tracks, monitors, and recovers overpayments eligible for recovery through combined efforts of the multiple VA Offices.
+Financial Services Center
+The Financial Services Center, a franchise fund (fee-for-service) organization, provides required recovery audit services to Veterans Health Administration, National Cemetery Administration, Veterans Benefits Administration, and VA Staff Offices. VA Staff Offices include but are not limited to the Office of Inspector General, Office of Acquisition Logistics and Construction, Office of Human Resources &amp; Administration, Office of Information Technology, and Office of Management.
+The Financial Services Center’s recovery audit program is focused on detection and recovery of overpayments for each program the Financial Services Center services that expends $1 million or more annually. The Financial Services Center reviews current and past payments in database portals to identify and recover improper payments such as duplicate payments, payments made in the incorrect amount, unapplied credits, etc. The Financial Services Center works with its customers to process bills of collection for identified improper payments.
+Office of Inspector General
+For improper payments that originate with payroll services, the Office of Inspector General works with two Office of Management and Budget Human Resources Lines of Business Shared Services Providers for its recovery audit requirements: the Bureau of Fiscal Services (Department of Treasury/Bureau of Fiscal Services), and the National Finance Center (Department of Agriculture/National Finance Center). Payroll overpayments and debt can arise for a variety of reasons including salary overpayments due to corrected timecards or personnel actions, debts arising from health and life insurance premiums or “buy backs” of employee leave, and administrative debts at the request of the agency.  The Bureau of Fiscal Services will automatically recalculate employee pay to recover overpayments related to corrected timecards and personnel actions. This process includes a Notification of Salary Overpayment to current employees and a Demand for Payment Notice to separated employees. The National Finance Center leads recovery efforts for overpayments that arise for all other reasons. If these efforts are unsuccessful, the debt is transferred to the United States Department of Treasury debt management for collection.
+Office of Revolving Funds
+The Office of Revolving Funds collaborates with the Office of Inspector General to perform recovery audits on VA's Supply Fund program. The Office of Inspector General identifies an overpayment and a bill of collection is then prepared by the Office of Revolving Funds with appropriate terms of collection. If the vendor chooses to dispute the bill of collection VA will work towards appropriate resolution.</t>
+  </si>
+  <si>
+    <t>The DoD Payment Recovery Audit (PRA) program is the Department’s overall plan for risk analysis and the performance of payment recovery audits. PRA’s are reviews and analyses of program accounting and financial records, supporting documentation, and other pertinent information supporting its payments; and, it is, designed specifically, to identify overpayments. It is through this system of internal controls surrounding the payments that assists in resolving the erroneous non-intentional monetary loss of Department dollars. The Department also utilizes collaborative working groups and enhanced specific reports that are disseminated to the responsible Component for the identification, validation and potential corrective actions for the trends of overpayment types if necessary.</t>
+  </si>
+  <si>
+    <t>A significant percentage of the Department's overpayments results from disallowed costs identified through grant audits. Other overpayments result from control deficiencies or errors in processing invoices.</t>
+  </si>
+  <si>
+    <t>The top root causes of UI improper payments for Payment Integrity Information Act (PIIA) 2022 (July 1, 2021 through June 30, 2022), were: Benefit Year Earnings (BYE), Separation Issues, and Other Eligibility improper payments (which includes the Identity Theft cause code).  The frequency and complexity of fraud attacks against state unemployment programs increased significantly during the COVID-19 pandemic. State UI systems were targeted by sophisticated and organized fraud, perpetrated by domestic and international criminal organizations. Fraud schemes continue to evolve to circumvent prevention and detection tools and strategies implemented by states. ETA and state UI agencies continue to work collaboratively with the Department’s Office of Inspector General (OIG) and refer cases of UI fraud, waste, abuse, mismanagement, and misconduct to the Department’s OIG for investigation and prosecution.
+ETA remains fully committed to reducing IPs and combatting fraud in the UI programs and continues to make UI program integrity a top agency priority. ETA develops, updates, and oversees implementation of a robust and dynamic UI Integrity Strategic Plan, which continuously evolves and includes innovative strategies to address emerging fraud schemes, prevent and reduce UI improper payments, and recover benefits that were overpaid. ETA’s FY 2022 efforts included providing guidance, technical assistance, and funding to support states in combatting fraud and reducing IP based on the top root causes of UI improper payments. ETA also invested in developing new and enhancing existing tools, datasets, and resources and made these available to aid states in more quickly identifying potential IP and fraud. For more information on the top root causes of UI improper payments and ETA’s UI integrity strategies and actions in FY 2022, see the FY 2022 UI Integrity Strategic Plan - https://oui.doleta.gov/unemploy/integrity_plan.asp</t>
+  </si>
+  <si>
+    <t>Grant payments continue to represent the greatest proportion of overpayments identified through the recovery audit.  DOT attributes the cause for grant-related overpayments to administrative errors made by entities external to the Department.  Over the course of FY 2021 and FY 2022, DOT has sought to conduct quantitative improper payment risk assessments (Phase 1) of COVID relief payments along with our annual estimates (Phase 2). The reviews reinforce DOT program oversight controls over relief funds administered by grant recipients and provide targeted actions for identified errors. The recovery audit provides an additional layer of detective controls to assess and confirm whether DOT’s improper payments remain within tolerable ranges.</t>
+  </si>
+  <si>
+    <t>Overpayments arise from various categories.  For example, it may be missing documentation, incorrect invoice amounts, eligibility, incomplete certifications, etc. The FCC looks at the various categories of overpayments and then determine whether stronger controls would help prevent the overpayments.</t>
+  </si>
+  <si>
+    <t>The overpayments were for two travelers, one who overestimated their parking amount and the other was paid for lodging taxes which were credited due to tax exemption.</t>
+  </si>
+  <si>
+    <t>Condition 1: The payment of real estate taxes in most leases is designed to be a passthrough from the landlord’s real estate tax bill.  The landlord pays the taxing authority and GSA pays the landlord for its share based on percentage occupancy of the building.  The real estate payment is incorporated into the GSA annual rent payment.  If the actual taxes are more than the amount paid through rent, GSA owes the landlord the difference.  If the actual taxes are less than the amount paid through rent, the landlord owes GSA the difference.  Recoveries arise when Lessor fails to report either of these two scenarios by not sending GSA the appropriate tax bills.    
+Resolution 1: GSA has established agencywide procedures to perform annual reviews of all leases when the landlord does not send in taxes.  These procedures have significantly decreased improper payments in this area in the last 4 years.
+Condition 2: There are several variables that can cause overpayments at the start up of a lease such as broker commission credits, free rent credits, and credits for holdover payments on a preceding lease, etc.  The overpayments exist if these credits are not entered in the billing system (REXUS) or not properly transferred from the billing system to the payment system (Pegasys).
+Resolution 2: Checklists have been developed in GSA's Regions to ensure that all credits are entered into the billing system (REXUS).  Also, in July of 2020, the REXUS to Pegasys interface automatically transfers data from REXUS to Pegasys so that it is no longer a manual process of entering credit data for leases into Pegasys which has helped reduce errors.</t>
+  </si>
+  <si>
+    <t>Recovery auditors conduct data analysis and review medical records to determine if what was billed and paid was accurate.  Typically these claims are chosen because of data analysis conducted based on the prior year improper payment rate data.  HHS uses RAC findings to prevent future improper payments through improvements to program operations, publication of detailed information in newsletters, implementation of local and/or national system edits, and other activities.</t>
+  </si>
+  <si>
+    <t>For internal offsets, over-claimed amounts (negative claims) occur when the mortgagee owes FHA.  The Single-Family Claims Branch (SFCB) sends billing letters to lenders for the excess amounts claimed and tracks the receivables using the Accounts Receivables Sub-system (ARS). Receivables are established in SFCB’s ARS and identified by an FHA case number. Each FHA case number is further identified by Section of the Act (which is linked to the appropriate fund) and endorsement date. This later date identifies the cohort year. The Holder of record to which the claim funds were originally disbursed is identified in ARS as the debtor, by default. When the receivable is subsequently liquidated by funds remitted by a Mortgagee or by offset, the collected amount is posted to the previously identified FHA case number, Section of the Act, and cohort year.
+If a payment is not received from a lender within 90 days, the receivable is offset against subsequent claims by the lender until the full amount of the receivable is satisfied. If a receivable is not satisfied within 120-150 days, it is referred to the FOC in Albany, NY for enforced collection actions. At that time, the FOC officially confirms acceptance of the transfer of an aged delinquent debt, and that receivables have been removed from the ARS with the notation that it has been referred to the FOC for recovery.
+Another avenue by which improper payments are recaptured is through Post Claim Reviews for title II Single Family Insurance Claims.  A statistical sample of settled claims is reviewed for compliance with FHA servicing and claim filing requirements. A report on findings, is prepared and issued to the individual mortgagee. Mortgagees can refute the findings by providing additional documents before a final report is issued. If the Mortgagee chooses to pay the monetary findings prior to HUD’s issuance of the final report, those funds are deposited to ARS, 
+which applies them to the Mortgage Insurance (MI) fund. Upon issuance of the final report, it is referred to the FOC which establishes it as a receivable and tracks it until paid in full. If a lender is overpaid on a Multifamily claim, the Multifamily Claims Branch will demand the overage back from the lender. If the lender fails to respond to their demands, the debt is referred to the FOC for collection. Lastly, for Treasury Cross-Servicing, the collection of generic debt is governed by the Debt Collection Improvement Act and HUD policies (Title I and Other Debt Collection Guidance 4740.2).  The Act requires federal agencies to refer eligible delinquent debts to Treasury (for Cross-Servicing and TOP) when the debt is 120 days delinquent.
+The Treasury’s TOP allows federal agencies to report delinquent non-tax debt to the Treasury’s Bureau of the Fiscal Service (BFS).  BFS performs computer matching with disbursement data and processes an offset when an appropriate match is determined. After referral, Treasury and its private collection agencies are responsible for contacting the debtor to collect the payment of the debt. The Treasury’s Cross-Servicing is a process used by BFS to refer the debt collection to a private collection agency, among other actions, to collect delinquent debts on behalf of Federal Agencies.
+The FOC’s recapture process establishes receivables in DCAMS and issues a demand notice to the debtor(s).  If the debt remains unpaid, DCAMS issues a “Notice of Intent” warning regarding enforced collection measures and informs the debtor regarding their due process rights. DCAMS automatically reports information to credit bureaus and CAIVRS. Penalty and administrative cost charges are also automatically assessed if warranted.
+If the debt remains unpaid, it is referred to Treasury (within 180 days) for offset via the government-wide TOP and for direct collection action by Treasury and Treasury contracted private collection agencies. Treasury also initiates referral to the Department of Justice (DOJ) for civil litigation and/or initiates Administrative Wage Garnishment (AWG) action if they deem such action to be appropriate.
+If Treasury’s Cross-Servicing action is not successful, Treasury “returns” the debt to the FOC. If older than two years, the receivable is written-off and the case is reclassified “currently not collectible.” The FOC keeps the case open if offset via TOP appears fruitful or if other collection measures are applicable (e.g., AWG action by HUD). Otherwise, the FOC terminates collection action, closes the case, and the system issues an IRS Form 1099C “Cancellation of Debt,” the following January if appropriate. Write-off, Termination, close-out, and 1099C issuance can also occur at any point in the above collection cycle if determined appropriate (e.g., debtor is discharged as bankrupt).
+Collections from debtors to HUD go to the Treasury Lockbox Network or Pay.gov. Collections from debtors to Treasury or DOJ come to HUD via interagency transfer (i.e., Intra-Governmental Payment and Collection (IPAC)). No matter the route, all payments are posted to the receivable in DCAMS.</t>
+  </si>
+  <si>
+    <t>There are no conditions known to OSC management that give rise to overpayments.</t>
+  </si>
+  <si>
+    <t>Clerical errors, calculation errors, technical errors, systems errors</t>
+  </si>
+  <si>
+    <t>Conditions arose from duplicate payments.</t>
+  </si>
+  <si>
+    <t>Many of Treasury's overpayments are travel or payroll related. These overpayments include issues such as corrected timecards, FEGLI corrections, duplicate cash awards, incorrect travel vouchers etc. Treasury also had contract overpayments which include duplicate amounts or incorrect amounts. Many of these overpayments were identified and recovered through post payment audits.</t>
+  </si>
+  <si>
+    <t>Overpayments identified in recovery audits are predominantly due to duplicate payments, non-compliance with contract billing requirements on federal supply schedule contracts, corrected timecards or personnel actions, processing dependency claims and due process, and discrepancies involving beneficiaries' income. These conditions are being resolved by implementing corrective actions utilizing mitigation strategies and corrective actions that are appropriate to the severity of the error. Examples include education and increased automation meant to identify and stop duplicate payments before they are made.</t>
+  </si>
+  <si>
+    <t>Internal recovery activities performed by DHS include, but are not limited to, grant and contract closeout processes, PIIA testing, self-reporting by vendors, duplicate payment reviews, usage of Do Not Pay capabilities and monitoring, etc.</t>
+  </si>
+  <si>
+    <t>The agency has not identified any improper payments so no additional action was required.</t>
+  </si>
+  <si>
+    <t>The Military Pay PRA incorporates all salary, benefits and other compensation related entitlements for all Service Members serving on Active Duty, Reserve and National Guard. Irrespective of actual assignment, the Service Members Branch handles Military Pay. For example, a Service Member assigned to a Combatant Command or Defense Agency; the Parent Military Branch is responsible for the Service Members pay. The Defense Finance and Accounting Service (DFAS) make these payments. The Military Branch coupled with DFAS relies heavily on their internal control process for pre and post payment reviews, entitlement verifications, reconciling management notices, Pay Record Accessibility audit, self-assessment program, and focus metrics program.
+The Department’s Civilian Pay PRA incorporates all salary, benefits and other compensation related entitlements for Department Civilians. The Civilian Pay process is dependent upon the built in internal controls for accuracy and timely distribution. The Department has an internal control structure in place for testing time and attendance that provides reasonable assurance that the hours worked, hours in pay status, and hours absent are properly recorded.
+The DoD Travel Pay, PRA program incorporates all of the payments made by DFAS, in support of the Military Branches, Combatant Commands and Defense Agencies for Service Members and Civilian Employees for mission required temporary and permanent travel- and/or transportation-related expenses. The Department through DFAS uses a variety of pre and post payment internal controls to identify, prevent and recoup travel overpayments.
+The Commercial Pay, PRA program is subject to all of the payments sent to Contractors and Vendors who provided various services and or delivered the required goods as outlined in the agreement or contract. The primary objective of the Commercial Pay Payment Recapture/Recovery Audit program is to recoup all monetary loss associated with payment made to outside Vendors and Contractors. The Department PRA Commercial Pay activities focuses on reporting and correcting any type of monetary loss. As part of the Department’s overall system of internal controls, any overpayments that have been identified in sampled items for the PIIA Compliance Audit are reported to the DoD Component where the transaction originated. The process is similar to when overpayments are discovered through different PIIA audits, reviews and reports. Regardless of the identification source of the overpayment, the Department actively pursues all available methods for recouping erroneous overpayments as part of the overarching PRA program.
+DFAS is the sole service provider for the processing and payroll of the Retired and Annuitant populations (R&amp;A) for the Department. DFAS is at the forefront of ensuring the appropriate controls are in place to combat and assist in the mitigation of risk for potential erroneous or improper payments. Based upon the guidance from the Department, DFAS R&amp;A quickly worked to identify and ascertain their processes that are in place to detect, identify and recoup any erroneous payments through its multiple payroll areas. DFAS is well postured to continue to identify the risks associated with payment recapture activities and implement checks and balances as a need arises.
+The U.S. Army Corps of Engineers (USACE) Finance Center (UFC) disburses all of the travel and commercial payments for USACE. USACE discovers overpayments through the contract closeout process, through routine audits and supplemented by the PIIA audit process. The USACE Finance Center Debt Management Office performs the necessary actions to recoup the payment once the overpayment is identified and the bill is created.
+The Military Health Benefits PRA program administered and managed by the Defense Health Agency (DHA). The TRICARE program provides healthcare services to 9.4 million beneficiaries. These refunds represent overpayments recovered as a result of payment errors identified through the compliance review process, refunds occurring in the course of routine healthcare claims processing, healthcare claim adjustments or corrections as identified by civilian providers or TRICARE beneficiaries and claim corrections as the result of internal post-payment audits conducted by private sector.</t>
+  </si>
+  <si>
+    <t>In FY 2022, the DOI had $28,061.41 million in outlays for all programs or activities that expend $1 million or more annually. For efforts conducted outside of payment recapture audits, DOI identified $4.41 million or .02 percent in overpayments and recovered $6.17 million or .02 percent. The sources used to identify the overpayments and recovered amounts were self-reported data gathered through Department Office and Bureau internal control reviews and single audit reports. In FY 2023, DOI will continue its efforts to recapture the balance identified but not recaptured in FY 2022.</t>
+  </si>
+  <si>
+    <t>Only OUI has determined that a recovery audit program is cost effective. 
+OUI reports the dollar amount of overpayments recovered through recovery audit during the reporting period as being used for the original purpose.  Any state UI dollars recovered are returned to state UI trust funds for use for the original purpose.  Any federal unemployment compensation funds are returned to Treasury for use for the original purpose.  OUI does not capture data on recovery aging to determine amounts determined uncollectable for overpayments identified in prior reporting periods.
+Other recovery activity data provided here is based on OCFO action. Component agencies may conduct recovery activities which are not tracked.</t>
+  </si>
+  <si>
+    <t>Please note that the EAC does conduct regular reviews and audits of its grants program through FFR and Progress Report reviews and audit resolution during which if any unknown payments are identified, they would be further pursued for recapture as appropriate.</t>
+  </si>
+  <si>
+    <t>The EEOC will continue to monitor its improper payments across all programs and activities that it administers and assess whether implementing payment recapture audits for each program is cost-effective.</t>
+  </si>
+  <si>
+    <t>The EPA uses various methods to recover improper payments. For Grants, Contracts, and Commodities, collection notices  are sent out via Pay.gov. In-service Payroll improper payments are rectified through salary offsets or supplements. Post-service collection recoveries are initiated through letter and/or email with repayments directed to Pay.gov. For Clean Water and Drinking Water State Revolving Funds recoveries typically occur through off-sets from future payments.</t>
+  </si>
+  <si>
+    <t>Given the small size of our agency (total budget of $84.8M for FY2022), that we don't have individual programs with outlays over $10M, and our low-risk status for improper payments, recovery audits are not cost-effective. Our improper payments are only .07% of total outlays for FY2022. We work to recover all identified improper payments in conjunction with our service provider. The benefits of any recovered amounts would not exceed the cost of a recovery audit program.</t>
+  </si>
+  <si>
+    <t>GSA identified possible improper payments related to a contract modification effective in FY 22. This contract modification incorporates a negotiated agreement between GSA and the vendor for $5,802,885. GSA needs to research contract documents to determine if the negotiated amount relates to a potential improper payment or proper payment.</t>
+  </si>
+  <si>
+    <t>HHS has a risk-based strategy to implement PIIA’s recovery auditing provisions.  Specifically, HHS focuses on implementing recovery audit programs in Medicare and providing a framework for states to implement recovery audit programs in Medicaid, which together account for most of HHS’s outlays.  HHS is progressing in recovering overpayments in Medicare and Medicaid and, most importantly, implementing corrective actions to prevent improper payments, as described in PaymentAccuracy.gov's program-specific pages and the FY 2022 HHS Agency Financial Report (available at www.hhs.gov/afr).  HHS considers lessons learned from these experiences as it implements this requirement.  
+While Medicare RACs are overseen and administered by CMS, Medicaid RACs are state-run programs. CMS does not collect as much information for this recovery source as the Medicare RACs.  Thus, some information presented in the recovery audit section may only account for information from a subset of the Department's RAC programs.
+For Medicaid FFS RACs, the amount recovered also subtracted amounts overturned on appeal or underpayments restored.</t>
+  </si>
+  <si>
+    <t>Annually, NASA performs an internal review of Overpayments Outside of Recovery Audit as a mechanism to identify and analyze the cause and amount of improper payments and total amounts recovered. The scope of the review includes cost-type and fixed priced contracts. The review includes an Agency-wide data call to allow for reporting of Agency identified overpayments and collections of improper payments. The data call is sent to the Office of the Chief Financial Officer organizations at NASA Centers, Office of Inspector General (OIG), Office of Procurement and the Headquarters Office of the Chief Financial Officer Policy &amp; Grants Division. Examples of activities included in reporting are Agency post-payment review/audits, single audit, and self-reported overpayments, which include OIG investigation settlements.</t>
+  </si>
+  <si>
+    <t>NEH has a 100% recovery rate of any improper payments identified.  NEH did not identify any improper payments in FY22.</t>
+  </si>
+  <si>
+    <t>NSF recovery activities include but are not limited to: resolution of questioned costs identified in audit reports, agency post-payment reviews, and other remittances received during normal payment operations.  Not all remittances that NSF receives through normal payment operations are considered overpayments as defined in PIIA.  However, NSF includes all of these operational remittances in its overpayments identified and recovered totals for completeness.  For audit resolution and agency post-payment reviews, NSF uses electronic notices/letters to identify and recover overpayments identified through these specific recovery activities.</t>
+  </si>
+  <si>
+    <t>Potential improper payments are subjected to further analysis based on the amount of the payment, the nature of the potential error, and other risk factors to determine whether amounts are due to PBGC. For Benefit Payments, PBGC has established procedures to recapture overpayments through electronic
+reclamation and debt collection agreements. PBGC forwards most of its benefit overpayment debts to the Centralized Receivables Service (CRS) of the Treasury Department to serve as its debt collection agent. CRS has the capability to enter into installment repayment agreements and offsets against other federal benefits. In some cases, recapture of payments may not be sought based on demonstration that a participant is experiencing financial hardship or other reasons. Other PBGC payment streams also have procedures in place to collect overpayments</t>
+  </si>
+  <si>
+    <t>The SBA makes every effort to recover improper payments identified during their improper payment review process.  This recovery effort is independent of the recapture audit process, which can be deemed costly and ineffective.  The SBA's process for recovering improper payments commences at the program office where the improper payments are identified.  The agency efforts to recapture improper payments are discussed by program or activity below.
+(a) Loan Program Purchases - Overpayments identified in the improper payments’ reviews are recaptured from the lender. The Quality Control staff tracks and collects any monetary overpayment. In some instances, the loan is referred to the Guaranty Denial Team for further action. Determination of a course of action is made on a case-by-case basis, depending on the specific details of the reason for the improper payment. Refer to Part I above for corrective action plans to prevent future improper payments.
+7(a) Loan Program Approvals and 504 Loan Guaranty Approvals - Overpayments recaptured outside payment recapture audits are not applicable to 7(a) loan guaranty approval and 504 loan approval as no payment is made at the time of approval. Improper payments identified through the annual improper payment reviews in 7(a) and 504 loan guaranty approvals are resolved through obtaining additional documentation, loan modification, or cancellation of the loan. Improper payments identified as a result of the FY 2021 PIIA reviews have been resolved through obtaining additional documentation, or cancellation or reduction of the loan guaranty and/or referral to other offices within the Office of Capital Access, as appropriate. Determination of a course of action is made on a case-by-case basis, which varies substantially depending on the circumstances of the loan approval and lender’s authority.
+Disaster Direct Loan Program - Overpayments are the result of the borrower receiving both an SBA loan and insurance payments or other benefits as a result of the disaster. If the duplication of benefit is recognized prior to the final disbursement, the loan amount is modified to reflect a lower amount and no repayment is required. If the duplication of benefit is identified after the final disbursement of the loan, then the borrower is given 30 days to provide evidence to prove that the disaster loan was not over-disbursed. For example, the borrower can provide documentation demonstrating that insurance funds received did not duplicate the disaster loan purpose. If the borrower has not provided the appropriate evidence within the 30-day period, a demand is made for the over-disbursed funds. Collection efforts continue at the Disaster loan servicing centers, but if these efforts fail, the borrower will still be liable for the over-disbursed amount in the form of monthly payments in accordance with the loan agreement. Thus, any actual loss is the cost of funds related to the over disbursement.
+COVID-Economic Injury Disaster Loan (EIDL) (COVID-EIDL) - Improper payments are generally the result of loan documentation errors.  Loan documentation legally obligates the recipient of a disaster loan to pay back the entire loan amount whether or not the loan contains any improper payments.  Therefore, improper payments are not recovered upon discovery but realized as the borrower makes each payment on the loan.  
+Economic Injury Disaster Loan Emergency Assistance (Advance) (EIDL Advance) - SBA is developing a plan to assess the Emergency EIDL Advances.  SBA will demand repayment for EIDL Advances identified as improper.  SBA will explore available options to remedy cases, including recovery of funds by offset, referral to OIG’s Division of Investigations, or providing supporting documentation where appropriate.  
+Paycheck Protection Program Loans - Overpayments are the result of the borrower receiving a PPP loan in an amount that (1) exceeds the borrower’s eligibility, (2) that cannot supported through documentation, or (3) that was not used for purposes permitted by statute or guidance.  In its review of the loan, if SBA determines that the loan is not eligible for forgiveness (in whole or in part), the borrower must begin paying principal and interest.</t>
+  </si>
+  <si>
+    <t>In making the determination, that recovery audits were not cost effective, the SEC considered its low improper payment rate based on testing conducted over several years.</t>
+  </si>
+  <si>
+    <t>Historically, our remittance process was a largely manual workload handled by the Mid-Atlantic Program Service Center (MATPSC).  The MATPSC remittance process requires a method of payment (check, money order, debit or credit card) and a corresponding payment coupon necessary to update a debtor’s record.  In fiscal year (FY) 2021, as part of the Debt Management Product, we implemented several improvements to our remittance process.  These enhancements now account for nearly 50 percent of our remittance activity.
+In January 2021, we partnered with the Department of the Treasury’s (Treasury) Pay.gov team to implement our first online repayment option for Old-Age, Survivors, and Disability Insurance beneficiaries and Supplemental Security Income recipients to repay benefit overpayments via credit or debit card and automated clearing house (ACH); i.e., a checking or savings account.  In FY 2022, we processed 456,000 remittances and collected $92 million through Pay.gov.
+Also, in January 2021, we partnered with Treasury to use U.S. Bank, a financial agent for Treasury, to implement a lockbox service to assist with our paper remittance processing efforts at the MATPSC.  In FY 2022, we processed 264,000 remittances and collected $69 million through the lockbox service.
+In July 2021, we implemented Online Bill Pay (OLBP), allowing debtors to make a one-time or recurring ACH draft from a bank account using a personal computer or mobile phone.  Prior to this implementation, OLBP remittances defaulted to paper checks.  In FY 2022, we processed 18,000 remittances and collected $2.5 million through OLBP.</t>
+  </si>
+  <si>
+    <t>Unknown payments identified in FY 2022 = $.063M</t>
+  </si>
+  <si>
+    <t>USAID continues to monitor and assess the improper payment reviews to ensure appropriate integrity and accuracy of payments such as sampling transactions, data analysis techniques and self-reports from mission overseas and Washington.  There is a low improper payment rate for the fiscal year 2022.</t>
+  </si>
+  <si>
+    <t>Most of the USITC's overpayments are payments to employees, such as unrecovered FICA tax that was not withheld and the employee subsequently left the agency. Some of these employees have paid the amounts, and we continue to contact those that have not. Even then these amounts are in the $5,000 range. We have occasionally (but not recently) overpaid a vendor or paid the wrong one, but these amounts were in the $10,000 range. When we cannot recover the payment we refer the vendor to the Treasury offset program.</t>
+  </si>
+  <si>
+    <t>Although VA has instituted payment integrity controls meant to identify overpayments before they occur, not all overpayments can be prevented. Therefore, VA implements appropriate recovery activities and audits based on the specifics of the program. The majority of VA's programs conduct recovery audits versus recovery activities.
+VA's recovery response is provided at the agency level based on an aggregate of program specific data. As a result, individual program responses may not be reflective of the overall agency response. For example, while VA responded yes to recovery activities, only 21 of 88 programs performed recovery activities in addition to recovery audits. In addition, some recoveries identified by Office of Management and Budget implementation guidance as activities versus recovery audits are so minimal throughout a fiscal year that it would not be cost beneficial to break these out and track separately, therefore, these are included in recovery audit reporting and recovery disposition aligns with recovery audit disposition requirements. Examples include overpayments identified during annual Payment Integrity Information Act of 2019 testing for programs reporting improper and unknown payments, recoveries from Qui Tam cases where VA does not receive notification from the Department of Justice that these recoveries were from a Qui Tam case, and some self-reported overpayments. Also, although the majority of VA’s programs are part of the Recovery Audit program facilitated by the Financial Services Center that has a recovery target of 80%, some programs have differing targets dependent upon specifics related to their programs.
+In addition, VA totals for the disposition of funds are able to be reconciled to the recovery audit amount for the reporting period; however, recovery audit overpayments identified in the current reporting period that remain outstanding for zero to six months or six months to one year may not reconcile to the difference in the amount identified and amount recovered for the current reporting period. This is a result of the amount recovered in the current reporting period including overpayments identified both within the reporting period and from prior reporting periods.</t>
+  </si>
+  <si>
+    <t>The Department’s uncollectable amounts is based primarily on a Military Commander or Senior Executive Leader authorized forgiven amounts for a particular Service Member, Civilian or Veteran. Overarching reasons include debt processing error, VA waiver, erroneous payments, financial hardship, injustice, and deceased Service Members.</t>
+  </si>
+  <si>
+    <t>The Department has a high rate of recovery. Nonetheless, in some instances, overpayments identified through recovery audit activities are deemed not collectible.</t>
+  </si>
+  <si>
+    <t>State UI programs may write off an overpayment when they determine it as uncollectable. This means that all reasonable collection efforts have been exhausted and the overpayment has been officially written off and/or authorized for removal from the active accounts receivable file and transferred to suspense (no further action to be taken).</t>
+  </si>
+  <si>
+    <t>Travel debt has a $25.00 threshold for collection. Any amount beneath the threshold is written off.</t>
+  </si>
+  <si>
+    <t>Some examples of a reason a collection is not possible are:  lease termination, company is bankrupt, or a change in ownership.  In these cases, the debt is referred to the Treasury for collection after 120 days.</t>
+  </si>
+  <si>
+    <t>The cost of recovery outweighs the amount to be recovered. The time elapsed between occurrence and discovery is often too great and with high staff turnover the ability to recover funds through external measures takes longer and is not fully effective.</t>
+  </si>
+  <si>
+    <t>Most of the amounts determined to not be collectable were due to travel or payroll improper payments. In the case of the Office of DC Pensions, individual debt cases deemed uncollectible after thorough reviews resulted in determinations to cease active collection actions.</t>
+  </si>
+  <si>
+    <t>VA reported overpayments identified in recovery audits that were determined not collectable. After exhausting all avenues to recover identified overpayments, including offsets, referrals to the Debt Management Center, and referrals to the Treasury Offset Program, the reported amount has been deemed uncollectable. For example, unique circumstances for approved waivers may determine the debt uncollectable.</t>
+  </si>
+  <si>
+    <t>Recovery Audits: Rates and Dispositions</t>
+  </si>
+  <si>
+    <t>Recovery Activities</t>
+  </si>
+  <si>
+    <t>ara2_1*</t>
+  </si>
+  <si>
+    <t>*overflow text from responses exceeding the character limit in the original response cell. ara2_1 &amp; [ara2_1]Provide a minimum of 2-4 sentences explaining the methods used by the agency to recover Improper Payments identified in recovery AUDITS. (Unit- Free-Text)</t>
+  </si>
+  <si>
+    <t>...that time, the FOC officially confirms acceptance of the transfer of an aged delinquent debt, and that receivables have been removed from the ARS with the notation that it has been referred to the FOC for recovery.
+Another avenue by which improper payments are recaptured is through Post Claim Reviews for title II Single Family Insurance Claims. A statistical sample of settled claims is reviewed for compliance with FHA servicing and claim filing requirements. A report on findings, is prepared and issued to the individual mortgagee. Mortgagees can refute the findings by providing additional documents before a final report is issued. If the Mortgagee chooses to pay the monetary findings prior to HUD’s issuance of the final report, those funds are deposited to ARS,
+which applies them to the Mortgage Insurance (MI) fund. Upon issuance of the final report, it is referred to the FOC which establishes it as a receivable and tracks it until paid in full. If a lender is overpaid on a Multifamily claim, the Multifamily Claims Branch will demand the overage back from the lender. If the lender fails to respond to their demands, the debt is referred to the FOC for collection. Lastly, for Treasury Cross-Servicing, the collection of generic debt is governed by the Debt Collection Improvement Act and HUD policies (Title I and Other Debt Collection Guidance 4740.2). The Act requires federal agencies to refer eligible delinquent debts to Treasury (for Cross-Servicing and TOP) when the debt is 120 days delinquent.
+The Treasury’s TOP allows federal agencies to report delinquent non-tax debt to the Treasury’s Bureau of the Fiscal Service (BFS). BFS performs computer matching with disbursement data and processes an offset when an appropriate match is determined. After referral, Treasury and its private collection agencies are responsible for contacting the debtor to collect the payment of the debt. The Treasury’s Cross-Servicing is a process used by BFS to refer the debt collection to a private collection agency, among other actions, to collect delinquent debts on behalf of Federal Agencies.
+The FOC’s recapture process establishes receivables in DCAMS and issues a demand notice to the debtor(s). If the debt remains unpaid, DCAMS issues a “Notice of Intent” warning regarding enforced collection measures and informs the debtor regarding their due process rights. DCAMS automatically reports information to credit bureaus and CAIVRS. Penalty and administrative cost charges are also automatically assessed if warranted.
+If the debt remains unpaid, it is referred to Treasury (within 180 days) for offset via the government-wide TOP and for direct collection action by Treasury and Treasury contracted private collection agencies. Treasury also initiates referral to the Department of Justice (DOJ) for civil litigation and/or initiates Administrative Wage Garnishment (AWG) action if they deem such action to be appropriate.
+If Treasury’s Cross-Servicing action is not successful, Treasury “returns” the debt to the FOC. If older than two years, the receivable is written-off and the case is reclassified “currently not collectible.” The FOC keeps the case open if offset via TOP appears fruitful or if other collection measures are applicable (e.g., AWG action by HUD). Otherwise, the FOC terminates collection action, closes the case, and the system issues an IRS Form 1099C “Cancellation of Debt,” the following January if appropriate. Write-off, Termination, close-out, and 1099C issuance can also occur at any point in the above collection cycle if determined appropriate (e.g., debtor is discharged as bankrupt).
+Collections from debtors to HUD go to the Treasury Lockbox Network or Pay.gov. Collections from debtors to Treasury or DOJ come to HUD via interagency transfer (i.e., Intra-Governmental Payment and Collection (IPAC)). No matter the route, all payments are posted to the receivable in DCAMS.</t>
+  </si>
+  <si>
     <t>(Community Development Block Grant (CDBG) –Disaster Relief Appropriation Act (DRAA) Sandy – CPD)
 The CPD Community Development Block Grant – DRAA-Sandy program monitors disaster recovery activities for Federally declared disaster arepas affected by Hurricane Sandy. The grantee submits a quarterly performance report using the Disaster Recovery Grant Reporting (DRGR) system that is reviewed by CPD field offices or HUD headquarters. The performance reports are used to review the grant expenditures and accomplishments for all CDBG-DR funded activities. The grantee also uses the DRGR system to submit vouchers and drawdown funds. After a voucher is created and submitted by a grantee Drawdown Requester, the voucher line items must be reviewed and approved by the grantee Drawdown Approver. If a line item is approved, it is either sent to the Line of Credit Control System (LOCCS) for processing, or, if the grant drawdown threshold of $5 million has been reached, it is sent to HUD for review and approval before it can be submitted to LOCCS. CPD also monitors the grantee’s efforts to prevent the duplication of benefits and ensure programmatic compliance. 
 CPD’s program exhibit 34-1, Guide for Review of Financial Management and Audits, is designed to monitor non-federal entity’s compliance with requirements Subparts D and F of 2 CFR part 200, Uniform Administrative Requirements, Cost Principles, and Audit Requirements for Federal Awards, except for cost allowability, procurement, and equipment. The exhibits located in Chapter 6 of the CPD Monitoring Handbook, serve the purpose of capturing improper payments identified in the program file-level reviews during on-site or remote monitoring. If any improper payments are identified the reviewer must indicate on the monitoring exhibit the program area, amount, type of improper payment and the corrective action. The grantee is notified of any improper payments identified during the monitoring review at the exit conference. If the grantee is unable to provide documentation to resolve the improper payment, a finding will be issued in the Monitoring Report which is transmitted to the grantee within 90 days of the monitoring review. In most cases, CPD recaptures overpayments by offsetting future draws. If there are no remaining funds on the grant, HUD typically instructs the grantee to either repay funds from non-federal sources to their grant’s line of credit in LOCCS, or to Treasury’s account if the grant has closed or the funding availability period has expired. Additionally, CPD may also withhold additional funding until the overpayment has been recovered. 
@@ -1634,206 +1852,7 @@
 Under Title I and Other Debt Collection Guidance Handbook 4740.2, the Financial Operation Center (FOC) is primarily responsible for generic debt collection and customer service activities, including responding to debtor inquiries regarding pay-off, payment plans, compromises, disputes, and appeals. The debt referral package primarily consists of copies of legal documents, mortgages, deeds of trust, judgments and other recorded lien documents, lien assignment documents, repayment agreements, credit reports, correspondence to/from debtors, and compromise agreements and supporting documents.
 The Debt Collection Asset Management System (DCAMS) is the application used to support the generic debt collection process. DCAMS is designed to automatically send collection letters, report delinquent debt to credit bureaus and HUD’s Credit Alert Interactive Voice Response System (CAIVRS), assess penalties and administrative costs, and refer eligible debts to the Treasury Offset Program (TOP) and Cross-Servicing. Based on predefined criteria and the status of that case as reflected in DCAMS data fields (not later than 180 days after the demand letter), DCAMS is consistently updated to prevent improper referral for TOP offset.
 For internal offsets, over-claimed amounts (negative claims) occur when the mortgagee owes FHA. The Single-Family Claims Branch (SFCB) sends billing letters to lenders for the excess amounts claimed and tracks the receivables using the Accounts Receivables Sub-system (ARS). Receivables are established in SFCB’s ARS and identified by an FHA case number. Each FHA case number is further identified by Section of the Act (which is linked to the appropriate fund) and endorsement date. This later date identifies the cohort year. The Holder of record to which the claim funds were originally disbursed is identified in ARS as the debtor, by default. When the receivable is subsequently liquidated by funds remitted by a Mortgagee or by offset, the collected amount is posted to the previously identified FHA case number, Section of the Act, and cohort year.
-If a payment is not received from a lender within 90 days, the receivable is offset against subsequent claims by the lender until the full amount of the receivable is satisfied. If a receivable is not satisfied within 120-150 days, it is referred to the FOC in Albany, NY for enforced collection actions. At th</t>
-  </si>
-  <si>
-    <t>OSC monitors various aspects of its financial activities throughout the year, including spot reviews of the agency's transit subsidy usage, analysis of expected payroll and benefits against the actual payroll and benefits, etc., and addresses any instances where overpayments are identified.</t>
-  </si>
-  <si>
-    <t>Bills of collection, offset of future payments, Treasury CRS</t>
-  </si>
-  <si>
-    <t>Recapture audits were performed internally instead of by a external contractor.</t>
-  </si>
-  <si>
-    <t>Invoices processed through the Invoice Processing Platform (IPP) are subject to a monthly post payment audit of 10% of the total paid IPP invoices for that month.  Invoices not processed through the Invoice Processing Platform (IPP) in excess of $2,500.00 are subject to secondary review before being paid.  Invoices under $2,500.00 are subject to review through statistical sampling procedures.  Travel vouchers processed through the Concur Government Edition (CGE) travel system are subject to a post payment audit based on a random sample of all reimbursements under $2,500.   All payments of $2,500.00 and higher are excluded from the population. These payments require a 100% post payment audit review. Relocation vouchers processed through the MoveLINQ system are subject to 100% pre-payment audit and review.   For payment customers, once the vouchers have been pre-audited and approved for payment, they are interfaced to the Oracle the financial system through which they are paid.   
-The DNP portal implementation has provided a way for our procurement and payable offices to review vendor files prior to disbursement.  It has also given us an opportunity to review the monthly payment file results to identify any improper payments made to a vendor in the DNP portal.</t>
-  </si>
-  <si>
-    <t>VA has established recovery audits in a manner that maximizes efficiency; therefore, many programs' payments are audited for overpayments that can be recovered using the same processes and procedures. At VA, these audits are performed in five major areas: Veterans Health Administration for several unique programs providing health care, Veterans Benefits Administration for benefit programs where the Financial Services Center in Austin, Texas does not process their payments, the Financial Services Center which provides recovery audits for all payments it processes which includes Veterans Health Administration payments, some Veterans Benefits Administration payments, National Cemetery Administration payments, and VA's Staff Offices (for example, Office of Information Technology, Office of Management, and the Office of Human Resources &amp; Administration/Operations, Security &amp; Preparedness), as well as specific recovery audits performed by the Office of Inspector General's additional shared service providers for payroll and Supply Fund payments in the Office of Revolving Fund. These are discussed in more detail below.
-Veterans Health Administration
-Veterans Health Administration is operationalizing a recovery audit contract which will audit claims from FY 2018 through FY 2023 for Civilian Health and Medical Program of the Department of Veterans Affairs, Veterans Health Administration Spina Bifida Health Care, and VA Community Care programs. The review includes inpatient claims paid under the following authorities: 38 U.S.C. § 1703 (authorized care); 38 U.S.C. § 1728 (service connected unauthorized care); and 38 U.S.C. § 1725 (non-service connected emergency care) and will test to ensure the care rendered is in compliance with the authorization/referral; was reimbursed based on the appropriate methodology; and that the medical records support the diagnostic related group billed for the services.
-Veterans Benefits Administration
-Veterans Benefits Administration uses a combination of quality reviews and payment reviews to identify possible duplicates and overpayments. The majority of Veterans Benefits Administration programs perform quality reviews on randomly selected cases that ensure eligibility determinations, proper case processing, and payment accuracy. For all other programs, Veterans Benefits Administration performs payment reviews to identify potential duplicate payments and other potential improper payments. Veterans Benefits Administration tracks, monitors, and recovers overpayments eligible for recovery through combined efforts of the multiple VA Offices.
-Financial Services Center
-The Financial Services Center, a franchise fund (fee-for-service) organization, provides required recovery audit services to Veterans Health Administration, National Cemetery Administration, Veterans Benefits Administration, and VA Staff Offices. VA Staff Offices include but are not limited to the Office of Inspector General, Office of Acquisition Logistics and Construction, Office of Human Resources &amp; Administration, Office of Information Technology, and Office of Management.
-The Financial Services Center’s recovery audit program is focused on detection and recovery of overpayments for each program the Financial Services Center services that expends $1 million or more annually. The Financial Services Center reviews current and past payments in database portals to identify and recover improper payments such as duplicate payments, payments made in the incorrect amount, unapplied credits, etc. The Financial Services Center works with its customers to process bills of collection for identified improper payments.
-Office of Inspector General
-For improper payments that originate with payroll services, the Office of Inspector General works with two Office of Management and Budget Human Resources Lines of Business Shared Services Providers for its recovery audit requirements: the Bureau of Fiscal Services (Department of Treasury/Bureau of Fiscal Services), and the National Finance Center (Department of Agriculture/National Finance Center). Payroll overpayments and debt can arise for a variety of reasons including salary overpayments due to corrected timecards or personnel actions, debts arising from health and life insurance premiums or “buy backs” of employee leave, and administrative debts at the request of the agency.  The Bureau of Fiscal Services will automatically recalculate employee pay to recover overpayments related to corrected timecards and personnel actions. This process includes a Notification of Salary Overpayment to current employees and a Demand for Payment Notice to separated employees. The National Finance Center leads recovery efforts for overpayments that arise for all other reasons. If these efforts are unsuccessful, the debt is transferred to the United States Department of Treasury debt management for collection.
-Office of Revolving Funds
-The Office of Revolving Funds collaborates with the Office of Inspector General to perform recovery audits on VA's Supply Fund program. The Office of Inspector General identifies an overpayment and a bill of collection is then prepared by the Office of Revolving Funds with appropriate terms of collection. If the vendor chooses to dispute the bill of collection VA will work towards appropriate resolution.</t>
-  </si>
-  <si>
-    <t>The DoD Payment Recovery Audit (PRA) program is the Department’s overall plan for risk analysis and the performance of payment recovery audits. PRA’s are reviews and analyses of program accounting and financial records, supporting documentation, and other pertinent information supporting its payments; and, it is, designed specifically, to identify overpayments. It is through this system of internal controls surrounding the payments that assists in resolving the erroneous non-intentional monetary loss of Department dollars. The Department also utilizes collaborative working groups and enhanced specific reports that are disseminated to the responsible Component for the identification, validation and potential corrective actions for the trends of overpayment types if necessary.</t>
-  </si>
-  <si>
-    <t>A significant percentage of the Department's overpayments results from disallowed costs identified through grant audits. Other overpayments result from control deficiencies or errors in processing invoices.</t>
-  </si>
-  <si>
-    <t>The top root causes of UI improper payments for Payment Integrity Information Act (PIIA) 2022 (July 1, 2021 through June 30, 2022), were: Benefit Year Earnings (BYE), Separation Issues, and Other Eligibility improper payments (which includes the Identity Theft cause code).  The frequency and complexity of fraud attacks against state unemployment programs increased significantly during the COVID-19 pandemic. State UI systems were targeted by sophisticated and organized fraud, perpetrated by domestic and international criminal organizations. Fraud schemes continue to evolve to circumvent prevention and detection tools and strategies implemented by states. ETA and state UI agencies continue to work collaboratively with the Department’s Office of Inspector General (OIG) and refer cases of UI fraud, waste, abuse, mismanagement, and misconduct to the Department’s OIG for investigation and prosecution.
-ETA remains fully committed to reducing IPs and combatting fraud in the UI programs and continues to make UI program integrity a top agency priority. ETA develops, updates, and oversees implementation of a robust and dynamic UI Integrity Strategic Plan, which continuously evolves and includes innovative strategies to address emerging fraud schemes, prevent and reduce UI improper payments, and recover benefits that were overpaid. ETA’s FY 2022 efforts included providing guidance, technical assistance, and funding to support states in combatting fraud and reducing IP based on the top root causes of UI improper payments. ETA also invested in developing new and enhancing existing tools, datasets, and resources and made these available to aid states in more quickly identifying potential IP and fraud. For more information on the top root causes of UI improper payments and ETA’s UI integrity strategies and actions in FY 2022, see the FY 2022 UI Integrity Strategic Plan - https://oui.doleta.gov/unemploy/integrity_plan.asp</t>
-  </si>
-  <si>
-    <t>Grant payments continue to represent the greatest proportion of overpayments identified through the recovery audit.  DOT attributes the cause for grant-related overpayments to administrative errors made by entities external to the Department.  Over the course of FY 2021 and FY 2022, DOT has sought to conduct quantitative improper payment risk assessments (Phase 1) of COVID relief payments along with our annual estimates (Phase 2). The reviews reinforce DOT program oversight controls over relief funds administered by grant recipients and provide targeted actions for identified errors. The recovery audit provides an additional layer of detective controls to assess and confirm whether DOT’s improper payments remain within tolerable ranges.</t>
-  </si>
-  <si>
-    <t>Overpayments arise from various categories.  For example, it may be missing documentation, incorrect invoice amounts, eligibility, incomplete certifications, etc. The FCC looks at the various categories of overpayments and then determine whether stronger controls would help prevent the overpayments.</t>
-  </si>
-  <si>
-    <t>The overpayments were for two travelers, one who overestimated their parking amount and the other was paid for lodging taxes which were credited due to tax exemption.</t>
-  </si>
-  <si>
-    <t>Condition 1: The payment of real estate taxes in most leases is designed to be a passthrough from the landlord’s real estate tax bill.  The landlord pays the taxing authority and GSA pays the landlord for its share based on percentage occupancy of the building.  The real estate payment is incorporated into the GSA annual rent payment.  If the actual taxes are more than the amount paid through rent, GSA owes the landlord the difference.  If the actual taxes are less than the amount paid through rent, the landlord owes GSA the difference.  Recoveries arise when Lessor fails to report either of these two scenarios by not sending GSA the appropriate tax bills.    
-Resolution 1: GSA has established agencywide procedures to perform annual reviews of all leases when the landlord does not send in taxes.  These procedures have significantly decreased improper payments in this area in the last 4 years.
-Condition 2: There are several variables that can cause overpayments at the start up of a lease such as broker commission credits, free rent credits, and credits for holdover payments on a preceding lease, etc.  The overpayments exist if these credits are not entered in the billing system (REXUS) or not properly transferred from the billing system to the payment system (Pegasys).
-Resolution 2: Checklists have been developed in GSA's Regions to ensure that all credits are entered into the billing system (REXUS).  Also, in July of 2020, the REXUS to Pegasys interface automatically transfers data from REXUS to Pegasys so that it is no longer a manual process of entering credit data for leases into Pegasys which has helped reduce errors.</t>
-  </si>
-  <si>
-    <t>Recovery auditors conduct data analysis and review medical records to determine if what was billed and paid was accurate.  Typically these claims are chosen because of data analysis conducted based on the prior year improper payment rate data.  HHS uses RAC findings to prevent future improper payments through improvements to program operations, publication of detailed information in newsletters, implementation of local and/or national system edits, and other activities.</t>
-  </si>
-  <si>
-    <t>For internal offsets, over-claimed amounts (negative claims) occur when the mortgagee owes FHA.  The Single-Family Claims Branch (SFCB) sends billing letters to lenders for the excess amounts claimed and tracks the receivables using the Accounts Receivables Sub-system (ARS). Receivables are established in SFCB’s ARS and identified by an FHA case number. Each FHA case number is further identified by Section of the Act (which is linked to the appropriate fund) and endorsement date. This later date identifies the cohort year. The Holder of record to which the claim funds were originally disbursed is identified in ARS as the debtor, by default. When the receivable is subsequently liquidated by funds remitted by a Mortgagee or by offset, the collected amount is posted to the previously identified FHA case number, Section of the Act, and cohort year.
-If a payment is not received from a lender within 90 days, the receivable is offset against subsequent claims by the lender until the full amount of the receivable is satisfied. If a receivable is not satisfied within 120-150 days, it is referred to the FOC in Albany, NY for enforced collection actions. At that time, the FOC officially confirms acceptance of the transfer of an aged delinquent debt, and that receivables have been removed from the ARS with the notation that it has been referred to the FOC for recovery.
-Another avenue by which improper payments are recaptured is through Post Claim Reviews for title II Single Family Insurance Claims.  A statistical sample of settled claims is reviewed for compliance with FHA servicing and claim filing requirements. A report on findings, is prepared and issued to the individual mortgagee. Mortgagees can refute the findings by providing additional documents before a final report is issued. If the Mortgagee chooses to pay the monetary findings prior to HUD’s issuance of the final report, those funds are deposited to ARS, 
-which applies them to the Mortgage Insurance (MI) fund. Upon issuance of the final report, it is referred to the FOC which establishes it as a receivable and tracks it until paid in full. If a lender is overpaid on a Multifamily claim, the Multifamily Claims Branch will demand the overage back from the lender. If the lender fails to respond to their demands, the debt is referred to the FOC for collection. Lastly, for Treasury Cross-Servicing, the collection of generic debt is governed by the Debt Collection Improvement Act and HUD policies (Title I and Other Debt Collection Guidance 4740.2).  The Act requires federal agencies to refer eligible delinquent debts to Treasury (for Cross-Servicing and TOP) when the debt is 120 days delinquent.
-The Treasury’s TOP allows federal agencies to report delinquent non-tax debt to the Treasury’s Bureau of the Fiscal Service (BFS).  BFS performs computer matching with disbursement data and processes an offset when an appropriate match is determined. After referral, Treasury and its private collection agencies are responsible for contacting the debtor to collect the payment of the debt. The Treasury’s Cross-Servicing is a process used by BFS to refer the debt collection to a private collection agency, among other actions, to collect delinquent debts on behalf of Federal Agencies.
-The FOC’s recapture process establishes receivables in DCAMS and issues a demand notice to the debtor(s).  If the debt remains unpaid, DCAMS issues a “Notice of Intent” warning regarding enforced collection measures and informs the debtor regarding their due process rights. DCAMS automatically reports information to credit bureaus and CAIVRS. Penalty and administrative cost charges are also automatically assessed if warranted.
-If the debt remains unpaid, it is referred to Treasury (within 180 days) for offset via the government-wide TOP and for direct collection action by Treasury and Treasury contracted private collection agencies. Treasury also initiates referral to the Department of Justice (DOJ) for civil litigation and/or initiates Administrative Wage Garnishment (AWG) action if they deem such action to be appropriate.
-If Treasury’s Cross-Servicing action is not successful, Treasury “returns” the debt to the FOC. If older than two years, the receivable is written-off and the case is reclassified “currently not collectible.” The FOC keeps the case open if offset via TOP appears fruitful or if other collection measures are applicable (e.g., AWG action by HUD). Otherwise, the FOC terminates collection action, closes the case, and the system issues an IRS Form 1099C “Cancellation of Debt,” the following January if appropriate. Write-off, Termination, close-out, and 1099C issuance can also occur at any point in the above collection cycle if determined appropriate (e.g., debtor is discharged as bankrupt).
-Collections from debtors to HUD go to the Treasury Lockbox Network or Pay.gov. Collections from debtors to Treasury or DOJ come to HUD via interagency transfer (i.e., Intra-Governmental Payment and Collection (IPAC)). No matter the route, all payments are posted to the receivable in DCAMS.</t>
-  </si>
-  <si>
-    <t>There are no conditions known to OSC management that give rise to overpayments.</t>
-  </si>
-  <si>
-    <t>Clerical errors, calculation errors, technical errors, systems errors</t>
-  </si>
-  <si>
-    <t>Conditions arose from duplicate payments.</t>
-  </si>
-  <si>
-    <t>Many of Treasury's overpayments are travel or payroll related. These overpayments include issues such as corrected timecards, FEGLI corrections, duplicate cash awards, incorrect travel vouchers etc. Treasury also had contract overpayments which include duplicate amounts or incorrect amounts. Many of these overpayments were identified and recovered through post payment audits.</t>
-  </si>
-  <si>
-    <t>Overpayments identified in recovery audits are predominantly due to duplicate payments, non-compliance with contract billing requirements on federal supply schedule contracts, corrected timecards or personnel actions, processing dependency claims and due process, and discrepancies involving beneficiaries' income. These conditions are being resolved by implementing corrective actions utilizing mitigation strategies and corrective actions that are appropriate to the severity of the error. Examples include education and increased automation meant to identify and stop duplicate payments before they are made.</t>
-  </si>
-  <si>
-    <t>Internal recovery activities performed by DHS include, but are not limited to, grant and contract closeout processes, PIIA testing, self-reporting by vendors, duplicate payment reviews, usage of Do Not Pay capabilities and monitoring, etc.</t>
-  </si>
-  <si>
-    <t>The agency has not identified any improper payments so no additional action was required.</t>
-  </si>
-  <si>
-    <t>The Military Pay PRA incorporates all salary, benefits and other compensation related entitlements for all Service Members serving on Active Duty, Reserve and National Guard. Irrespective of actual assignment, the Service Members Branch handles Military Pay. For example, a Service Member assigned to a Combatant Command or Defense Agency; the Parent Military Branch is responsible for the Service Members pay. The Defense Finance and Accounting Service (DFAS) make these payments. The Military Branch coupled with DFAS relies heavily on their internal control process for pre and post payment reviews, entitlement verifications, reconciling management notices, Pay Record Accessibility audit, self-assessment program, and focus metrics program.
-The Department’s Civilian Pay PRA incorporates all salary, benefits and other compensation related entitlements for Department Civilians. The Civilian Pay process is dependent upon the built in internal controls for accuracy and timely distribution. The Department has an internal control structure in place for testing time and attendance that provides reasonable assurance that the hours worked, hours in pay status, and hours absent are properly recorded.
-The DoD Travel Pay, PRA program incorporates all of the payments made by DFAS, in support of the Military Branches, Combatant Commands and Defense Agencies for Service Members and Civilian Employees for mission required temporary and permanent travel- and/or transportation-related expenses. The Department through DFAS uses a variety of pre and post payment internal controls to identify, prevent and recoup travel overpayments.
-The Commercial Pay, PRA program is subject to all of the payments sent to Contractors and Vendors who provided various services and or delivered the required goods as outlined in the agreement or contract. The primary objective of the Commercial Pay Payment Recapture/Recovery Audit program is to recoup all monetary loss associated with payment made to outside Vendors and Contractors. The Department PRA Commercial Pay activities focuses on reporting and correcting any type of monetary loss. As part of the Department’s overall system of internal controls, any overpayments that have been identified in sampled items for the PIIA Compliance Audit are reported to the DoD Component where the transaction originated. The process is similar to when overpayments are discovered through different PIIA audits, reviews and reports. Regardless of the identification source of the overpayment, the Department actively pursues all available methods for recouping erroneous overpayments as part of the overarching PRA program.
-DFAS is the sole service provider for the processing and payroll of the Retired and Annuitant populations (R&amp;A) for the Department. DFAS is at the forefront of ensuring the appropriate controls are in place to combat and assist in the mitigation of risk for potential erroneous or improper payments. Based upon the guidance from the Department, DFAS R&amp;A quickly worked to identify and ascertain their processes that are in place to detect, identify and recoup any erroneous payments through its multiple payroll areas. DFAS is well postured to continue to identify the risks associated with payment recapture activities and implement checks and balances as a need arises.
-The U.S. Army Corps of Engineers (USACE) Finance Center (UFC) disburses all of the travel and commercial payments for USACE. USACE discovers overpayments through the contract closeout process, through routine audits and supplemented by the PIIA audit process. The USACE Finance Center Debt Management Office performs the necessary actions to recoup the payment once the overpayment is identified and the bill is created.
-The Military Health Benefits PRA program administered and managed by the Defense Health Agency (DHA). The TRICARE program provides healthcare services to 9.4 million beneficiaries. These refunds represent overpayments recovered as a result of payment errors identified through the compliance review process, refunds occurring in the course of routine healthcare claims processing, healthcare claim adjustments or corrections as identified by civilian providers or TRICARE beneficiaries and claim corrections as the result of internal post-payment audits conducted by private sector.</t>
-  </si>
-  <si>
-    <t>In FY 2022, the DOI had $28,061.41 million in outlays for all programs or activities that expend $1 million or more annually. For efforts conducted outside of payment recapture audits, DOI identified $4.41 million or .02 percent in overpayments and recovered $6.17 million or .02 percent. The sources used to identify the overpayments and recovered amounts were self-reported data gathered through Department Office and Bureau internal control reviews and single audit reports. In FY 2023, DOI will continue its efforts to recapture the balance identified but not recaptured in FY 2022.</t>
-  </si>
-  <si>
-    <t>Only OUI has determined that a recovery audit program is cost effective. 
-OUI reports the dollar amount of overpayments recovered through recovery audit during the reporting period as being used for the original purpose.  Any state UI dollars recovered are returned to state UI trust funds for use for the original purpose.  Any federal unemployment compensation funds are returned to Treasury for use for the original purpose.  OUI does not capture data on recovery aging to determine amounts determined uncollectable for overpayments identified in prior reporting periods.
-Other recovery activity data provided here is based on OCFO action. Component agencies may conduct recovery activities which are not tracked.</t>
-  </si>
-  <si>
-    <t>Please note that the EAC does conduct regular reviews and audits of its grants program through FFR and Progress Report reviews and audit resolution during which if any unknown payments are identified, they would be further pursued for recapture as appropriate.</t>
-  </si>
-  <si>
-    <t>The EEOC will continue to monitor its improper payments across all programs and activities that it administers and assess whether implementing payment recapture audits for each program is cost-effective.</t>
-  </si>
-  <si>
-    <t>The EPA uses various methods to recover improper payments. For Grants, Contracts, and Commodities, collection notices  are sent out via Pay.gov. In-service Payroll improper payments are rectified through salary offsets or supplements. Post-service collection recoveries are initiated through letter and/or email with repayments directed to Pay.gov. For Clean Water and Drinking Water State Revolving Funds recoveries typically occur through off-sets from future payments.</t>
-  </si>
-  <si>
-    <t>Given the small size of our agency (total budget of $84.8M for FY2022), that we don't have individual programs with outlays over $10M, and our low-risk status for improper payments, recovery audits are not cost-effective. Our improper payments are only .07% of total outlays for FY2022. We work to recover all identified improper payments in conjunction with our service provider. The benefits of any recovered amounts would not exceed the cost of a recovery audit program.</t>
-  </si>
-  <si>
-    <t>GSA identified possible improper payments related to a contract modification effective in FY 22. This contract modification incorporates a negotiated agreement between GSA and the vendor for $5,802,885. GSA needs to research contract documents to determine if the negotiated amount relates to a potential improper payment or proper payment.</t>
-  </si>
-  <si>
-    <t>HHS has a risk-based strategy to implement PIIA’s recovery auditing provisions.  Specifically, HHS focuses on implementing recovery audit programs in Medicare and providing a framework for states to implement recovery audit programs in Medicaid, which together account for most of HHS’s outlays.  HHS is progressing in recovering overpayments in Medicare and Medicaid and, most importantly, implementing corrective actions to prevent improper payments, as described in PaymentAccuracy.gov's program-specific pages and the FY 2022 HHS Agency Financial Report (available at www.hhs.gov/afr).  HHS considers lessons learned from these experiences as it implements this requirement.  
-While Medicare RACs are overseen and administered by CMS, Medicaid RACs are state-run programs. CMS does not collect as much information for this recovery source as the Medicare RACs.  Thus, some information presented in the recovery audit section may only account for information from a subset of the Department's RAC programs.
-For Medicaid FFS RACs, the amount recovered also subtracted amounts overturned on appeal or underpayments restored.</t>
-  </si>
-  <si>
-    <t>Annually, NASA performs an internal review of Overpayments Outside of Recovery Audit as a mechanism to identify and analyze the cause and amount of improper payments and total amounts recovered. The scope of the review includes cost-type and fixed priced contracts. The review includes an Agency-wide data call to allow for reporting of Agency identified overpayments and collections of improper payments. The data call is sent to the Office of the Chief Financial Officer organizations at NASA Centers, Office of Inspector General (OIG), Office of Procurement and the Headquarters Office of the Chief Financial Officer Policy &amp; Grants Division. Examples of activities included in reporting are Agency post-payment review/audits, single audit, and self-reported overpayments, which include OIG investigation settlements.</t>
-  </si>
-  <si>
-    <t>NEH has a 100% recovery rate of any improper payments identified.  NEH did not identify any improper payments in FY22.</t>
-  </si>
-  <si>
-    <t>NSF recovery activities include but are not limited to: resolution of questioned costs identified in audit reports, agency post-payment reviews, and other remittances received during normal payment operations.  Not all remittances that NSF receives through normal payment operations are considered overpayments as defined in PIIA.  However, NSF includes all of these operational remittances in its overpayments identified and recovered totals for completeness.  For audit resolution and agency post-payment reviews, NSF uses electronic notices/letters to identify and recover overpayments identified through these specific recovery activities.</t>
-  </si>
-  <si>
-    <t>Potential improper payments are subjected to further analysis based on the amount of the payment, the nature of the potential error, and other risk factors to determine whether amounts are due to PBGC. For Benefit Payments, PBGC has established procedures to recapture overpayments through electronic
-reclamation and debt collection agreements. PBGC forwards most of its benefit overpayment debts to the Centralized Receivables Service (CRS) of the Treasury Department to serve as its debt collection agent. CRS has the capability to enter into installment repayment agreements and offsets against other federal benefits. In some cases, recapture of payments may not be sought based on demonstration that a participant is experiencing financial hardship or other reasons. Other PBGC payment streams also have procedures in place to collect overpayments</t>
-  </si>
-  <si>
-    <t>The SBA makes every effort to recover improper payments identified during their improper payment review process.  This recovery effort is independent of the recapture audit process, which can be deemed costly and ineffective.  The SBA's process for recovering improper payments commences at the program office where the improper payments are identified.  The agency efforts to recapture improper payments are discussed by program or activity below.
-(a) Loan Program Purchases - Overpayments identified in the improper payments’ reviews are recaptured from the lender. The Quality Control staff tracks and collects any monetary overpayment. In some instances, the loan is referred to the Guaranty Denial Team for further action. Determination of a course of action is made on a case-by-case basis, depending on the specific details of the reason for the improper payment. Refer to Part I above for corrective action plans to prevent future improper payments.
-7(a) Loan Program Approvals and 504 Loan Guaranty Approvals - Overpayments recaptured outside payment recapture audits are not applicable to 7(a) loan guaranty approval and 504 loan approval as no payment is made at the time of approval. Improper payments identified through the annual improper payment reviews in 7(a) and 504 loan guaranty approvals are resolved through obtaining additional documentation, loan modification, or cancellation of the loan. Improper payments identified as a result of the FY 2021 PIIA reviews have been resolved through obtaining additional documentation, or cancellation or reduction of the loan guaranty and/or referral to other offices within the Office of Capital Access, as appropriate. Determination of a course of action is made on a case-by-case basis, which varies substantially depending on the circumstances of the loan approval and lender’s authority.
-Disaster Direct Loan Program - Overpayments are the result of the borrower receiving both an SBA loan and insurance payments or other benefits as a result of the disaster. If the duplication of benefit is recognized prior to the final disbursement, the loan amount is modified to reflect a lower amount and no repayment is required. If the duplication of benefit is identified after the final disbursement of the loan, then the borrower is given 30 days to provide evidence to prove that the disaster loan was not over-disbursed. For example, the borrower can provide documentation demonstrating that insurance funds received did not duplicate the disaster loan purpose. If the borrower has not provided the appropriate evidence within the 30-day period, a demand is made for the over-disbursed funds. Collection efforts continue at the Disaster loan servicing centers, but if these efforts fail, the borrower will still be liable for the over-disbursed amount in the form of monthly payments in accordance with the loan agreement. Thus, any actual loss is the cost of funds related to the over disbursement.
-COVID-Economic Injury Disaster Loan (EIDL) (COVID-EIDL) - Improper payments are generally the result of loan documentation errors.  Loan documentation legally obligates the recipient of a disaster loan to pay back the entire loan amount whether or not the loan contains any improper payments.  Therefore, improper payments are not recovered upon discovery but realized as the borrower makes each payment on the loan.  
-Economic Injury Disaster Loan Emergency Assistance (Advance) (EIDL Advance) - SBA is developing a plan to assess the Emergency EIDL Advances.  SBA will demand repayment for EIDL Advances identified as improper.  SBA will explore available options to remedy cases, including recovery of funds by offset, referral to OIG’s Division of Investigations, or providing supporting documentation where appropriate.  
-Paycheck Protection Program Loans - Overpayments are the result of the borrower receiving a PPP loan in an amount that (1) exceeds the borrower’s eligibility, (2) that cannot supported through documentation, or (3) that was not used for purposes permitted by statute or guidance.  In its review of the loan, if SBA determines that the loan is not eligible for forgiveness (in whole or in part), the borrower must begin paying principal and interest.</t>
-  </si>
-  <si>
-    <t>In making the determination, that recovery audits were not cost effective, the SEC considered its low improper payment rate based on testing conducted over several years.</t>
-  </si>
-  <si>
-    <t>Historically, our remittance process was a largely manual workload handled by the Mid-Atlantic Program Service Center (MATPSC).  The MATPSC remittance process requires a method of payment (check, money order, debit or credit card) and a corresponding payment coupon necessary to update a debtor’s record.  In fiscal year (FY) 2021, as part of the Debt Management Product, we implemented several improvements to our remittance process.  These enhancements now account for nearly 50 percent of our remittance activity.
-In January 2021, we partnered with the Department of the Treasury’s (Treasury) Pay.gov team to implement our first online repayment option for Old-Age, Survivors, and Disability Insurance beneficiaries and Supplemental Security Income recipients to repay benefit overpayments via credit or debit card and automated clearing house (ACH); i.e., a checking or savings account.  In FY 2022, we processed 456,000 remittances and collected $92 million through Pay.gov.
-Also, in January 2021, we partnered with Treasury to use U.S. Bank, a financial agent for Treasury, to implement a lockbox service to assist with our paper remittance processing efforts at the MATPSC.  In FY 2022, we processed 264,000 remittances and collected $69 million through the lockbox service.
-In July 2021, we implemented Online Bill Pay (OLBP), allowing debtors to make a one-time or recurring ACH draft from a bank account using a personal computer or mobile phone.  Prior to this implementation, OLBP remittances defaulted to paper checks.  In FY 2022, we processed 18,000 remittances and collected $2.5 million through OLBP.</t>
-  </si>
-  <si>
-    <t>Unknown payments identified in FY 2022 = $.063M</t>
-  </si>
-  <si>
-    <t>USAID continues to monitor and assess the improper payment reviews to ensure appropriate integrity and accuracy of payments such as sampling transactions, data analysis techniques and self-reports from mission overseas and Washington.  There is a low improper payment rate for the fiscal year 2022.</t>
-  </si>
-  <si>
-    <t>Most of the USITC's overpayments are payments to employees, such as unrecovered FICA tax that was not withheld and the employee subsequently left the agency. Some of these employees have paid the amounts, and we continue to contact those that have not. Even then these amounts are in the $5,000 range. We have occasionally (but not recently) overpaid a vendor or paid the wrong one, but these amounts were in the $10,000 range. When we cannot recover the payment we refer the vendor to the Treasury offset program.</t>
-  </si>
-  <si>
-    <t>Although VA has instituted payment integrity controls meant to identify overpayments before they occur, not all overpayments can be prevented. Therefore, VA implements appropriate recovery activities and audits based on the specifics of the program. The majority of VA's programs conduct recovery audits versus recovery activities.
-VA's recovery response is provided at the agency level based on an aggregate of program specific data. As a result, individual program responses may not be reflective of the overall agency response. For example, while VA responded yes to recovery activities, only 21 of 88 programs performed recovery activities in addition to recovery audits. In addition, some recoveries identified by Office of Management and Budget implementation guidance as activities versus recovery audits are so minimal throughout a fiscal year that it would not be cost beneficial to break these out and track separately, therefore, these are included in recovery audit reporting and recovery disposition aligns with recovery audit disposition requirements. Examples include overpayments identified during annual Payment Integrity Information Act of 2019 testing for programs reporting improper and unknown payments, recoveries from Qui Tam cases where VA does not receive notification from the Department of Justice that these recoveries were from a Qui Tam case, and some self-reported overpayments. Also, although the majority of VA’s programs are part of the Recovery Audit program facilitated by the Financial Services Center that has a recovery target of 80%, some programs have differing targets dependent upon specifics related to their programs.
-In addition, VA totals for the disposition of funds are able to be reconciled to the recovery audit amount for the reporting period; however, recovery audit overpayments identified in the current reporting period that remain outstanding for zero to six months or six months to one year may not reconcile to the difference in the amount identified and amount recovered for the current reporting period. This is a result of the amount recovered in the current reporting period including overpayments identified both within the reporting period and from prior reporting periods.</t>
-  </si>
-  <si>
-    <t>The Department’s uncollectable amounts is based primarily on a Military Commander or Senior Executive Leader authorized forgiven amounts for a particular Service Member, Civilian or Veteran. Overarching reasons include debt processing error, VA waiver, erroneous payments, financial hardship, injustice, and deceased Service Members.</t>
-  </si>
-  <si>
-    <t>The Department has a high rate of recovery. Nonetheless, in some instances, overpayments identified through recovery audit activities are deemed not collectible.</t>
-  </si>
-  <si>
-    <t>State UI programs may write off an overpayment when they determine it as uncollectable. This means that all reasonable collection efforts have been exhausted and the overpayment has been officially written off and/or authorized for removal from the active accounts receivable file and transferred to suspense (no further action to be taken).</t>
-  </si>
-  <si>
-    <t>Travel debt has a $25.00 threshold for collection. Any amount beneath the threshold is written off.</t>
-  </si>
-  <si>
-    <t>Some examples of a reason a collection is not possible are:  lease termination, company is bankrupt, or a change in ownership.  In these cases, the debt is referred to the Treasury for collection after 120 days.</t>
-  </si>
-  <si>
-    <t>The cost of recovery outweighs the amount to be recovered. The time elapsed between occurrence and discovery is often too great and with high staff turnover the ability to recover funds through external measures takes longer and is not fully effective.</t>
-  </si>
-  <si>
-    <t>Most of the amounts determined to not be collectable were due to travel or payroll improper payments. In the case of the Office of DC Pensions, individual debt cases deemed uncollectible after thorough reviews resulted in determinations to cease active collection actions.</t>
-  </si>
-  <si>
-    <t>VA reported overpayments identified in recovery audits that were determined not collectable. After exhausting all avenues to recover identified overpayments, including offsets, referrals to the Debt Management Center, and referrals to the Treasury Offset Program, the reported amount has been deemed uncollectable. For example, unique circumstances for approved waivers may determine the debt uncollectable.</t>
-  </si>
-  <si>
-    <t>Recovery Audits: Rates and Dispositions</t>
-  </si>
-  <si>
-    <t>Recovery Activities</t>
+If a payment is not received from a lender within 90 days, the receivable is offset against subsequent claims by the lender until the full amount of the receivable is satisfied. If a receivable is not satisfied within 120-150 days, it is referred to the FOC in Albany, NY for enforced collection actions. At...</t>
   </si>
 </sst>
 </file>
@@ -1916,7 +1935,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1948,7 +1967,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1969,9 +1994,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2009,7 +2034,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2115,7 +2140,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2257,7 +2282,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2265,77 +2290,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22618D3F-C01D-44CF-9330-E09D0B7E4ED3}">
-  <dimension ref="A1:AV56"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:AW56"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="12" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.45">
       <c r="C1" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
       <c r="L1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="M1" s="11" t="s">
-        <v>413</v>
-      </c>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="11"/>
-      <c r="T1" s="11"/>
-      <c r="U1" s="11"/>
-      <c r="V1" s="11"/>
-      <c r="W1" s="11"/>
-      <c r="X1" s="11"/>
-      <c r="Y1" s="10" t="s">
+      <c r="M1" s="12" t="s">
+        <v>412</v>
+      </c>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="Z1" s="10"/>
-      <c r="AA1" s="10"/>
-      <c r="AB1" s="10"/>
-      <c r="AC1" s="10"/>
-      <c r="AD1" s="10"/>
-      <c r="AE1" s="10" t="s">
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="13"/>
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="AF1" s="10"/>
-      <c r="AG1" s="10"/>
-      <c r="AH1" s="10"/>
-      <c r="AI1" s="10" t="s">
-        <v>412</v>
-      </c>
-      <c r="AJ1" s="10"/>
-      <c r="AK1" s="10"/>
-      <c r="AL1" s="10"/>
-      <c r="AM1" s="10"/>
-      <c r="AN1" s="10"/>
-      <c r="AO1" s="10"/>
-      <c r="AP1" s="10"/>
-      <c r="AQ1" s="10"/>
-      <c r="AR1" s="10"/>
-      <c r="AS1" s="10"/>
-      <c r="AT1" s="10"/>
-      <c r="AU1" s="10"/>
-      <c r="AV1" s="10"/>
+      <c r="AG1" s="11"/>
+      <c r="AH1" s="11"/>
+      <c r="AI1" s="11"/>
+      <c r="AJ1" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="AK1" s="11"/>
+      <c r="AL1" s="11"/>
+      <c r="AM1" s="11"/>
+      <c r="AN1" s="11"/>
+      <c r="AO1" s="11"/>
+      <c r="AP1" s="11"/>
+      <c r="AQ1" s="11"/>
+      <c r="AR1" s="11"/>
+      <c r="AS1" s="11"/>
+      <c r="AT1" s="11"/>
+      <c r="AU1" s="11"/>
+      <c r="AV1" s="11"/>
+      <c r="AW1" s="11"/>
     </row>
-    <row r="2" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.45">
       <c r="C2" s="2" t="s">
         <v>66</v>
       </c>
@@ -2408,74 +2434,77 @@
       <c r="Z2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="AA2" s="2" t="s">
+      <c r="AA2" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="AB2" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="AB2" s="2" t="s">
+      <c r="AC2" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="AC2" s="2" t="s">
+      <c r="AD2" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="AD2" s="2" t="s">
+      <c r="AE2" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="AE2" s="2" t="s">
+      <c r="AF2" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="AF2" s="2" t="s">
+      <c r="AG2" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="AG2" s="2" t="s">
+      <c r="AH2" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="AH2" s="2" t="s">
+      <c r="AI2" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="AI2" s="2" t="s">
+      <c r="AJ2" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="AJ2" s="2" t="s">
+      <c r="AK2" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="AK2" s="2" t="s">
+      <c r="AL2" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="AL2" s="2" t="s">
+      <c r="AM2" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="AM2" s="2" t="s">
+      <c r="AN2" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AN2" s="2" t="s">
+      <c r="AO2" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="AO2" s="2" t="s">
+      <c r="AP2" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="AP2" s="2" t="s">
+      <c r="AQ2" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="AQ2" s="2" t="s">
+      <c r="AR2" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="AR2" s="2" t="s">
+      <c r="AS2" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="AS2" s="2" t="s">
+      <c r="AT2" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="AT2" s="2" t="s">
+      <c r="AU2" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="AU2" s="2" t="s">
+      <c r="AV2" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="AV2" s="2" t="s">
+      <c r="AW2" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:48" s="6" customFormat="1" ht="152.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:49" s="6" customFormat="1" ht="152.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
         <v>151</v>
       </c>
@@ -2555,73 +2584,76 @@
         <v>103</v>
       </c>
       <c r="AA3" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="AB3" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="AB3" s="5" t="s">
+      <c r="AC3" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="AC3" s="5" t="s">
+      <c r="AD3" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="AD3" s="5" t="s">
+      <c r="AE3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="AE3" s="5" t="s">
+      <c r="AF3" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="AF3" s="5" t="s">
+      <c r="AG3" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="AG3" s="5" t="s">
+      <c r="AH3" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="AH3" s="5" t="s">
+      <c r="AI3" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="AI3" s="5" t="s">
+      <c r="AJ3" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="AJ3" s="5" t="s">
+      <c r="AK3" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="AK3" s="5" t="s">
+      <c r="AL3" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="AL3" s="5" t="s">
+      <c r="AM3" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="AM3" s="5" t="s">
+      <c r="AN3" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="AN3" s="5" t="s">
+      <c r="AO3" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="AO3" s="5" t="s">
+      <c r="AP3" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="AP3" s="5" t="s">
+      <c r="AQ3" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="AQ3" s="5" t="s">
+      <c r="AR3" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="AR3" s="5" t="s">
+      <c r="AS3" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="AS3" s="5" t="s">
+      <c r="AT3" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="AT3" s="5" t="s">
+      <c r="AU3" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="AU3" s="5" t="s">
+      <c r="AV3" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="AV3" s="5" t="s">
+      <c r="AW3" s="5" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="4" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -2684,10 +2716,10 @@
       <c r="AB4" s="3"/>
       <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
-      <c r="AE4" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF4" s="3"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
       <c r="AI4" s="3"/>
@@ -2704,8 +2736,9 @@
       <c r="AT4" s="3"/>
       <c r="AU4" s="3"/>
       <c r="AV4" s="3"/>
+      <c r="AW4" s="3"/>
     </row>
-    <row r="5" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -2776,10 +2809,10 @@
       <c r="AB5" s="3"/>
       <c r="AC5" s="3"/>
       <c r="AD5" s="3"/>
-      <c r="AE5" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF5" s="3"/>
+      <c r="AE5" s="3"/>
+      <c r="AF5" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
@@ -2796,8 +2829,9 @@
       <c r="AT5" s="3"/>
       <c r="AU5" s="3"/>
       <c r="AV5" s="3"/>
+      <c r="AW5" s="3"/>
     </row>
-    <row r="6" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
@@ -2876,10 +2910,10 @@
       <c r="AB6" s="3"/>
       <c r="AC6" s="3"/>
       <c r="AD6" s="3"/>
-      <c r="AE6" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF6" s="3"/>
+      <c r="AE6" s="3"/>
+      <c r="AF6" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
       <c r="AI6" s="3"/>
@@ -2896,8 +2930,9 @@
       <c r="AT6" s="3"/>
       <c r="AU6" s="3"/>
       <c r="AV6" s="3"/>
+      <c r="AW6" s="3"/>
     </row>
-    <row r="7" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -2958,15 +2993,15 @@
       <c r="AB7" s="3"/>
       <c r="AC7" s="3"/>
       <c r="AD7" s="3"/>
-      <c r="AE7" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF7" s="3"/>
+      <c r="AE7" s="3"/>
+      <c r="AF7" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG7" s="3"/>
-      <c r="AH7" s="3" t="s">
+      <c r="AH7" s="3"/>
+      <c r="AI7" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="AI7" s="3"/>
       <c r="AJ7" s="3"/>
       <c r="AK7" s="3"/>
       <c r="AL7" s="3"/>
@@ -2980,8 +3015,9 @@
       <c r="AT7" s="3"/>
       <c r="AU7" s="3"/>
       <c r="AV7" s="3"/>
+      <c r="AW7" s="3"/>
     </row>
-    <row r="8" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -3062,15 +3098,15 @@
       <c r="AB8" s="3"/>
       <c r="AC8" s="3"/>
       <c r="AD8" s="3"/>
-      <c r="AE8" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF8" s="3"/>
+      <c r="AE8" s="3"/>
+      <c r="AF8" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG8" s="3"/>
-      <c r="AH8" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="AI8" s="3"/>
+      <c r="AH8" s="3"/>
+      <c r="AI8" s="3" t="s">
+        <v>381</v>
+      </c>
       <c r="AJ8" s="3"/>
       <c r="AK8" s="3"/>
       <c r="AL8" s="3"/>
@@ -3084,8 +3120,9 @@
       <c r="AT8" s="3"/>
       <c r="AU8" s="3"/>
       <c r="AV8" s="3"/>
+      <c r="AW8" s="3"/>
     </row>
-    <row r="9" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
@@ -3138,15 +3175,15 @@
       <c r="AB9" s="3"/>
       <c r="AC9" s="3"/>
       <c r="AD9" s="3"/>
-      <c r="AE9" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF9" s="3"/>
+      <c r="AE9" s="3"/>
+      <c r="AF9" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG9" s="3"/>
-      <c r="AH9" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="AI9" s="3"/>
+      <c r="AH9" s="3"/>
+      <c r="AI9" s="3" t="s">
+        <v>382</v>
+      </c>
       <c r="AJ9" s="3"/>
       <c r="AK9" s="3"/>
       <c r="AL9" s="3"/>
@@ -3160,8 +3197,9 @@
       <c r="AT9" s="3"/>
       <c r="AU9" s="3"/>
       <c r="AV9" s="3"/>
+      <c r="AW9" s="3"/>
     </row>
-    <row r="10" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3240,10 +3278,10 @@
       <c r="AB10" s="3"/>
       <c r="AC10" s="3"/>
       <c r="AD10" s="3"/>
-      <c r="AE10" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF10" s="3"/>
+      <c r="AE10" s="3"/>
+      <c r="AF10" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
       <c r="AI10" s="3"/>
@@ -3260,8 +3298,9 @@
       <c r="AT10" s="3"/>
       <c r="AU10" s="3"/>
       <c r="AV10" s="3"/>
+      <c r="AW10" s="3"/>
     </row>
-    <row r="11" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
@@ -3334,74 +3373,75 @@
       <c r="Z11" s="3" t="s">
         <v>353</v>
       </c>
-      <c r="AA11" s="8">
+      <c r="AA11" s="3"/>
+      <c r="AB11" s="8">
         <v>1459.09</v>
       </c>
-      <c r="AB11" s="8">
+      <c r="AC11" s="8">
         <v>1393.97</v>
       </c>
-      <c r="AC11" s="8">
+      <c r="AD11" s="8">
         <v>78</v>
       </c>
-      <c r="AD11" s="3" t="s">
-        <v>368</v>
-      </c>
       <c r="AE11" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF11" s="8">
+        <v>367</v>
+      </c>
+      <c r="AF11" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AG11" s="8">
         <v>123.45</v>
       </c>
-      <c r="AG11" s="8">
-        <v>0</v>
-      </c>
-      <c r="AH11" s="3" t="s">
-        <v>384</v>
-      </c>
-      <c r="AI11" s="8">
+      <c r="AH11" s="8">
+        <v>0</v>
+      </c>
+      <c r="AI11" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="AJ11" s="8">
         <v>95.536944259777997</v>
       </c>
-      <c r="AJ11" s="8">
+      <c r="AK11" s="8">
         <v>12.64</v>
       </c>
-      <c r="AK11" s="8">
-        <v>0</v>
-      </c>
       <c r="AL11" s="8">
         <v>0</v>
       </c>
       <c r="AM11" s="8">
+        <v>0</v>
+      </c>
+      <c r="AN11" s="8">
         <v>1365.29</v>
       </c>
-      <c r="AN11" s="8">
-        <v>0</v>
-      </c>
       <c r="AO11" s="8">
+        <v>0</v>
+      </c>
+      <c r="AP11" s="8">
         <v>28.68</v>
       </c>
-      <c r="AP11" s="8">
-        <v>0</v>
-      </c>
       <c r="AQ11" s="8">
+        <v>0</v>
+      </c>
+      <c r="AR11" s="8">
         <v>160.4</v>
       </c>
-      <c r="AR11" s="8">
+      <c r="AS11" s="8">
         <v>141.84</v>
       </c>
-      <c r="AS11" s="3" t="s">
-        <v>404</v>
-      </c>
-      <c r="AT11" s="8">
+      <c r="AT11" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="AU11" s="8">
         <v>0.86629337463762002</v>
       </c>
-      <c r="AU11" s="8">
+      <c r="AV11" s="8">
         <v>302.24</v>
       </c>
-      <c r="AV11" s="8">
+      <c r="AW11" s="8">
         <v>20.71</v>
       </c>
     </row>
-    <row r="12" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
@@ -3480,10 +3520,10 @@
       <c r="AB12" s="3"/>
       <c r="AC12" s="3"/>
       <c r="AD12" s="3"/>
-      <c r="AE12" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF12" s="3"/>
+      <c r="AE12" s="3"/>
+      <c r="AF12" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
@@ -3500,8 +3540,9 @@
       <c r="AT12" s="3"/>
       <c r="AU12" s="3"/>
       <c r="AV12" s="3"/>
+      <c r="AW12" s="3"/>
     </row>
-    <row r="13" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>9</v>
       </c>
@@ -3582,15 +3623,15 @@
       <c r="AB13" s="3"/>
       <c r="AC13" s="3"/>
       <c r="AD13" s="3"/>
-      <c r="AE13" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF13" s="3"/>
+      <c r="AE13" s="3"/>
+      <c r="AF13" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG13" s="3"/>
-      <c r="AH13" s="3" t="s">
-        <v>385</v>
-      </c>
-      <c r="AI13" s="3"/>
+      <c r="AH13" s="3"/>
+      <c r="AI13" s="3" t="s">
+        <v>384</v>
+      </c>
       <c r="AJ13" s="3"/>
       <c r="AK13" s="3"/>
       <c r="AL13" s="3"/>
@@ -3604,8 +3645,9 @@
       <c r="AT13" s="3"/>
       <c r="AU13" s="3"/>
       <c r="AV13" s="3"/>
+      <c r="AW13" s="3"/>
     </row>
-    <row r="14" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
@@ -3680,46 +3722,44 @@
       <c r="Z14" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="AA14" s="8">
+      <c r="AA14" s="3"/>
+      <c r="AB14" s="8">
         <v>8.76</v>
       </c>
-      <c r="AB14" s="8">
+      <c r="AC14" s="8">
         <v>4.37</v>
       </c>
-      <c r="AC14" s="8">
+      <c r="AD14" s="8">
         <v>98</v>
       </c>
-      <c r="AD14" s="3" t="s">
-        <v>369</v>
-      </c>
       <c r="AE14" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF14" s="8">
+        <v>368</v>
+      </c>
+      <c r="AF14" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AG14" s="8">
         <v>1.53</v>
       </c>
-      <c r="AG14" s="8">
+      <c r="AH14" s="8">
         <v>0.03</v>
       </c>
-      <c r="AH14" s="3"/>
-      <c r="AI14" s="8">
+      <c r="AI14" s="3"/>
+      <c r="AJ14" s="8">
         <v>49.885844748857998</v>
       </c>
-      <c r="AJ14" s="8">
+      <c r="AK14" s="8">
         <v>0.03</v>
       </c>
-      <c r="AK14" s="8">
-        <v>0</v>
-      </c>
       <c r="AL14" s="8">
         <v>0</v>
       </c>
       <c r="AM14" s="8">
+        <v>0</v>
+      </c>
+      <c r="AN14" s="8">
         <v>4.37</v>
       </c>
-      <c r="AN14" s="8">
-        <v>0</v>
-      </c>
       <c r="AO14" s="8">
         <v>0</v>
       </c>
@@ -3727,25 +3767,28 @@
         <v>0</v>
       </c>
       <c r="AQ14" s="8">
+        <v>0</v>
+      </c>
+      <c r="AR14" s="8">
         <v>1.48</v>
       </c>
-      <c r="AR14" s="8">
+      <c r="AS14" s="8">
         <v>3.51</v>
       </c>
-      <c r="AS14" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="AT14" s="8">
+      <c r="AT14" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="AU14" s="8">
         <v>0.34246575342466001</v>
       </c>
-      <c r="AU14" s="8">
+      <c r="AV14" s="8">
         <v>4.99</v>
       </c>
-      <c r="AV14" s="8">
+      <c r="AW14" s="8">
         <v>56.963470319635</v>
       </c>
     </row>
-    <row r="15" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>11</v>
       </c>
@@ -3824,48 +3867,46 @@
       <c r="Z15" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="AA15" s="8">
+      <c r="AA15" s="3"/>
+      <c r="AB15" s="8">
         <v>4621.71</v>
       </c>
-      <c r="AB15" s="8">
+      <c r="AC15" s="8">
         <v>1110.78</v>
       </c>
-      <c r="AC15" s="8">
+      <c r="AD15" s="8">
         <v>68</v>
       </c>
-      <c r="AD15" s="3" t="s">
-        <v>370</v>
-      </c>
       <c r="AE15" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF15" s="8">
+        <v>369</v>
+      </c>
+      <c r="AF15" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AG15" s="8">
         <v>8812.34</v>
       </c>
-      <c r="AG15" s="8">
-        <v>0</v>
-      </c>
-      <c r="AH15" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="AI15" s="8">
+      <c r="AH15" s="8">
+        <v>0</v>
+      </c>
+      <c r="AI15" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="AJ15" s="8">
         <v>24.033961455825001</v>
       </c>
-      <c r="AJ15" s="8">
+      <c r="AK15" s="8">
         <v>508.94</v>
       </c>
-      <c r="AK15" s="8">
-        <v>0</v>
-      </c>
       <c r="AL15" s="8">
         <v>0</v>
       </c>
       <c r="AM15" s="8">
+        <v>0</v>
+      </c>
+      <c r="AN15" s="8">
         <v>1110.78</v>
       </c>
-      <c r="AN15" s="8">
-        <v>0</v>
-      </c>
       <c r="AO15" s="8">
         <v>0</v>
       </c>
@@ -3873,25 +3914,28 @@
         <v>0</v>
       </c>
       <c r="AQ15" s="8">
+        <v>0</v>
+      </c>
+      <c r="AR15" s="8">
         <v>6257.45</v>
       </c>
-      <c r="AR15" s="8">
+      <c r="AS15" s="8">
         <v>5948.52</v>
       </c>
-      <c r="AS15" s="3" t="s">
-        <v>406</v>
-      </c>
-      <c r="AT15" s="8">
+      <c r="AT15" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="AU15" s="8">
         <v>11.011941467552001</v>
       </c>
-      <c r="AU15" s="8">
+      <c r="AV15" s="8">
         <v>12205.97</v>
       </c>
-      <c r="AV15" s="8">
+      <c r="AW15" s="8">
         <v>264.10073327838001</v>
       </c>
     </row>
-    <row r="16" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>12</v>
       </c>
@@ -3964,34 +4008,32 @@
       <c r="Z16" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="AA16" s="8">
+      <c r="AA16" s="3"/>
+      <c r="AB16" s="8">
         <v>7.8154661000000001</v>
       </c>
-      <c r="AB16" s="8">
+      <c r="AC16" s="8">
         <v>7.6946615999999999</v>
       </c>
-      <c r="AC16" s="8">
+      <c r="AD16" s="8">
         <v>90</v>
       </c>
-      <c r="AD16" s="3" t="s">
-        <v>371</v>
-      </c>
       <c r="AE16" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF16" s="8">
+        <v>370</v>
+      </c>
+      <c r="AF16" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AG16" s="8">
         <v>6.50329801</v>
       </c>
-      <c r="AG16" s="8">
-        <v>0</v>
-      </c>
-      <c r="AH16" s="3"/>
-      <c r="AI16" s="8">
+      <c r="AH16" s="8">
+        <v>0</v>
+      </c>
+      <c r="AI16" s="3"/>
+      <c r="AJ16" s="8">
         <v>98.454289245781993</v>
       </c>
-      <c r="AJ16" s="8">
-        <v>0</v>
-      </c>
       <c r="AK16" s="8">
         <v>0</v>
       </c>
@@ -3999,11 +4041,11 @@
         <v>0</v>
       </c>
       <c r="AM16" s="8">
+        <v>0</v>
+      </c>
+      <c r="AN16" s="8">
         <v>7.6946615999999999</v>
       </c>
-      <c r="AN16" s="8">
-        <v>0</v>
-      </c>
       <c r="AO16" s="8">
         <v>0</v>
       </c>
@@ -4011,23 +4053,26 @@
         <v>0</v>
       </c>
       <c r="AQ16" s="8">
+        <v>0</v>
+      </c>
+      <c r="AR16" s="8">
         <v>0.1208045</v>
       </c>
-      <c r="AR16" s="8">
-        <v>0</v>
-      </c>
-      <c r="AS16" s="3"/>
-      <c r="AT16" s="8">
-        <v>0</v>
-      </c>
+      <c r="AS16" s="8">
+        <v>0</v>
+      </c>
+      <c r="AT16" s="3"/>
       <c r="AU16" s="8">
+        <v>0</v>
+      </c>
+      <c r="AV16" s="8">
         <v>0.1208045</v>
       </c>
-      <c r="AV16" s="8">
+      <c r="AW16" s="8">
         <v>1.5457107542185</v>
       </c>
     </row>
-    <row r="17" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>13</v>
       </c>
@@ -4076,27 +4121,27 @@
       <c r="Z17" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="AA17" s="8">
-        <v>0</v>
-      </c>
+      <c r="AA17" s="3"/>
       <c r="AB17" s="8">
         <v>0</v>
       </c>
       <c r="AC17" s="8">
         <v>0</v>
       </c>
-      <c r="AD17" s="3" t="s">
+      <c r="AD17" s="8">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="AE17" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF17" s="3"/>
+      <c r="AF17" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG17" s="3"/>
-      <c r="AH17" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="AI17" s="3"/>
+      <c r="AH17" s="3"/>
+      <c r="AI17" s="3" t="s">
+        <v>386</v>
+      </c>
       <c r="AJ17" s="3"/>
       <c r="AK17" s="3"/>
       <c r="AL17" s="3"/>
@@ -4104,20 +4149,21 @@
       <c r="AN17" s="3"/>
       <c r="AO17" s="3"/>
       <c r="AP17" s="3"/>
-      <c r="AQ17" s="8">
-        <v>0</v>
-      </c>
+      <c r="AQ17" s="3"/>
       <c r="AR17" s="8">
         <v>0</v>
       </c>
-      <c r="AS17" s="3"/>
+      <c r="AS17" s="8">
+        <v>0</v>
+      </c>
       <c r="AT17" s="3"/>
-      <c r="AU17" s="8">
-        <v>0</v>
-      </c>
-      <c r="AV17" s="3"/>
+      <c r="AU17" s="3"/>
+      <c r="AV17" s="8">
+        <v>0</v>
+      </c>
+      <c r="AW17" s="3"/>
     </row>
-    <row r="18" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>14</v>
       </c>
@@ -4196,10 +4242,10 @@
       <c r="AB18" s="3"/>
       <c r="AC18" s="3"/>
       <c r="AD18" s="3"/>
-      <c r="AE18" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF18" s="3"/>
+      <c r="AE18" s="3"/>
+      <c r="AF18" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
       <c r="AI18" s="3"/>
@@ -4216,8 +4262,9 @@
       <c r="AT18" s="3"/>
       <c r="AU18" s="3"/>
       <c r="AV18" s="3"/>
+      <c r="AW18" s="3"/>
     </row>
-    <row r="19" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>15</v>
       </c>
@@ -4280,15 +4327,15 @@
       <c r="AB19" s="3"/>
       <c r="AC19" s="3"/>
       <c r="AD19" s="3"/>
-      <c r="AE19" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF19" s="3"/>
+      <c r="AE19" s="3"/>
+      <c r="AF19" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG19" s="3"/>
-      <c r="AH19" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="AI19" s="3"/>
+      <c r="AH19" s="3"/>
+      <c r="AI19" s="3" t="s">
+        <v>387</v>
+      </c>
       <c r="AJ19" s="3"/>
       <c r="AK19" s="3"/>
       <c r="AL19" s="3"/>
@@ -4302,8 +4349,9 @@
       <c r="AT19" s="3"/>
       <c r="AU19" s="3"/>
       <c r="AV19" s="3"/>
+      <c r="AW19" s="3"/>
     </row>
-    <row r="20" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>16</v>
       </c>
@@ -4384,15 +4432,15 @@
       <c r="AB20" s="3"/>
       <c r="AC20" s="3"/>
       <c r="AD20" s="3"/>
-      <c r="AE20" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF20" s="3"/>
+      <c r="AE20" s="3"/>
+      <c r="AF20" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG20" s="3"/>
-      <c r="AH20" s="3" t="s">
-        <v>389</v>
-      </c>
-      <c r="AI20" s="3"/>
+      <c r="AH20" s="3"/>
+      <c r="AI20" s="3" t="s">
+        <v>388</v>
+      </c>
       <c r="AJ20" s="3"/>
       <c r="AK20" s="3"/>
       <c r="AL20" s="3"/>
@@ -4406,8 +4454,9 @@
       <c r="AT20" s="3"/>
       <c r="AU20" s="3"/>
       <c r="AV20" s="3"/>
+      <c r="AW20" s="3"/>
     </row>
-    <row r="21" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>17</v>
       </c>
@@ -4462,10 +4511,10 @@
       <c r="AB21" s="3"/>
       <c r="AC21" s="3"/>
       <c r="AD21" s="3"/>
-      <c r="AE21" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF21" s="3"/>
+      <c r="AE21" s="3"/>
+      <c r="AF21" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
       <c r="AI21" s="3"/>
@@ -4482,8 +4531,9 @@
       <c r="AT21" s="3"/>
       <c r="AU21" s="3"/>
       <c r="AV21" s="3"/>
+      <c r="AW21" s="3"/>
     </row>
-    <row r="22" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>18</v>
       </c>
@@ -4550,15 +4600,15 @@
       <c r="AB22" s="3"/>
       <c r="AC22" s="3"/>
       <c r="AD22" s="3"/>
-      <c r="AE22" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF22" s="3"/>
+      <c r="AE22" s="3"/>
+      <c r="AF22" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG22" s="3"/>
-      <c r="AH22" s="3" t="s">
-        <v>390</v>
-      </c>
-      <c r="AI22" s="3"/>
+      <c r="AH22" s="3"/>
+      <c r="AI22" s="3" t="s">
+        <v>389</v>
+      </c>
       <c r="AJ22" s="3"/>
       <c r="AK22" s="3"/>
       <c r="AL22" s="3"/>
@@ -4572,8 +4622,9 @@
       <c r="AT22" s="3"/>
       <c r="AU22" s="3"/>
       <c r="AV22" s="3"/>
+      <c r="AW22" s="3"/>
     </row>
-    <row r="23" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>19</v>
       </c>
@@ -4646,30 +4697,28 @@
       <c r="Z23" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="AA23" s="8">
+      <c r="AA23" s="3"/>
+      <c r="AB23" s="8">
         <v>8.0830000000000002</v>
       </c>
-      <c r="AB23" s="8">
+      <c r="AC23" s="8">
         <v>0.219</v>
       </c>
-      <c r="AC23" s="8">
+      <c r="AD23" s="8">
         <v>100</v>
       </c>
-      <c r="AD23" s="3" t="s">
-        <v>372</v>
-      </c>
       <c r="AE23" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF23" s="3"/>
+        <v>371</v>
+      </c>
+      <c r="AF23" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
-      <c r="AI23" s="8">
+      <c r="AI23" s="3"/>
+      <c r="AJ23" s="8">
         <v>2.7093900779414</v>
       </c>
-      <c r="AJ23" s="8">
-        <v>0</v>
-      </c>
       <c r="AK23" s="8">
         <v>0</v>
       </c>
@@ -4677,11 +4726,11 @@
         <v>0</v>
       </c>
       <c r="AM23" s="8">
+        <v>0</v>
+      </c>
+      <c r="AN23" s="8">
         <v>0.219</v>
       </c>
-      <c r="AN23" s="8">
-        <v>0</v>
-      </c>
       <c r="AO23" s="8">
         <v>0</v>
       </c>
@@ -4689,23 +4738,26 @@
         <v>0</v>
       </c>
       <c r="AQ23" s="8">
+        <v>0</v>
+      </c>
+      <c r="AR23" s="8">
         <v>7.1</v>
       </c>
-      <c r="AR23" s="8">
+      <c r="AS23" s="8">
         <v>0.314</v>
       </c>
-      <c r="AS23" s="3"/>
-      <c r="AT23" s="8">
-        <v>0</v>
-      </c>
+      <c r="AT23" s="3"/>
       <c r="AU23" s="8">
+        <v>0</v>
+      </c>
+      <c r="AV23" s="8">
         <v>7.4139999999999997</v>
       </c>
-      <c r="AV23" s="8">
+      <c r="AW23" s="8">
         <v>91.72</v>
       </c>
     </row>
-    <row r="24" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>20</v>
       </c>
@@ -4768,10 +4820,10 @@
       <c r="AB24" s="3"/>
       <c r="AC24" s="3"/>
       <c r="AD24" s="3"/>
-      <c r="AE24" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF24" s="3"/>
+      <c r="AE24" s="3"/>
+      <c r="AF24" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
       <c r="AI24" s="3"/>
@@ -4788,8 +4840,9 @@
       <c r="AT24" s="3"/>
       <c r="AU24" s="3"/>
       <c r="AV24" s="3"/>
+      <c r="AW24" s="3"/>
     </row>
-    <row r="25" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>21</v>
       </c>
@@ -4856,10 +4909,10 @@
       <c r="AB25" s="3"/>
       <c r="AC25" s="3"/>
       <c r="AD25" s="3"/>
-      <c r="AE25" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF25" s="3"/>
+      <c r="AE25" s="3"/>
+      <c r="AF25" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
       <c r="AI25" s="3"/>
@@ -4876,8 +4929,9 @@
       <c r="AT25" s="3"/>
       <c r="AU25" s="3"/>
       <c r="AV25" s="3"/>
+      <c r="AW25" s="3"/>
     </row>
-    <row r="26" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>22</v>
       </c>
@@ -4950,37 +5004,35 @@
       <c r="Z26" s="3" t="s">
         <v>359</v>
       </c>
-      <c r="AA26" s="8">
+      <c r="AA26" s="3"/>
+      <c r="AB26" s="8">
         <v>1.6880000000000001E-5</v>
       </c>
-      <c r="AB26" s="8">
-        <v>0</v>
-      </c>
       <c r="AC26" s="8">
+        <v>0</v>
+      </c>
+      <c r="AD26" s="8">
         <v>100</v>
       </c>
-      <c r="AD26" s="3" t="s">
-        <v>373</v>
-      </c>
       <c r="AE26" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF26" s="8">
-        <v>0</v>
+        <v>372</v>
+      </c>
+      <c r="AF26" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="AG26" s="8">
         <v>0</v>
       </c>
-      <c r="AH26" s="3"/>
-      <c r="AI26" s="8">
-        <v>0</v>
-      </c>
+      <c r="AH26" s="8">
+        <v>0</v>
+      </c>
+      <c r="AI26" s="3"/>
       <c r="AJ26" s="8">
+        <v>0</v>
+      </c>
+      <c r="AK26" s="8">
         <v>16.88</v>
       </c>
-      <c r="AK26" s="8">
-        <v>0</v>
-      </c>
       <c r="AL26" s="8">
         <v>0</v>
       </c>
@@ -5002,18 +5054,21 @@
       <c r="AR26" s="8">
         <v>0</v>
       </c>
-      <c r="AS26" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="AT26" s="8">
+      <c r="AS26" s="8">
+        <v>0</v>
+      </c>
+      <c r="AT26" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="AU26" s="8">
         <v>100000000</v>
       </c>
-      <c r="AU26" s="8">
-        <v>0</v>
-      </c>
-      <c r="AV26" s="3"/>
+      <c r="AV26" s="8">
+        <v>0</v>
+      </c>
+      <c r="AW26" s="3"/>
     </row>
-    <row r="27" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>23</v>
       </c>
@@ -5086,48 +5141,46 @@
       <c r="Z27" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="AA27" s="8">
+      <c r="AA27" s="3"/>
+      <c r="AB27" s="8">
         <v>3.55</v>
       </c>
-      <c r="AB27" s="8">
+      <c r="AC27" s="8">
         <v>3.46</v>
       </c>
-      <c r="AC27" s="8">
+      <c r="AD27" s="8">
         <v>80</v>
       </c>
-      <c r="AD27" s="3" t="s">
-        <v>374</v>
-      </c>
       <c r="AE27" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF27" s="8">
+        <v>373</v>
+      </c>
+      <c r="AF27" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AG27" s="8">
         <v>0.1</v>
       </c>
-      <c r="AG27" s="8">
+      <c r="AH27" s="8">
         <v>0.24</v>
       </c>
-      <c r="AH27" s="3" t="s">
-        <v>391</v>
-      </c>
-      <c r="AI27" s="8">
+      <c r="AI27" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="AJ27" s="8">
         <v>97.464788732393998</v>
       </c>
-      <c r="AJ27" s="8">
+      <c r="AK27" s="8">
         <v>0.01</v>
       </c>
-      <c r="AK27" s="8">
+      <c r="AL27" s="8">
         <v>0.83</v>
       </c>
-      <c r="AL27" s="8">
-        <v>0</v>
-      </c>
       <c r="AM27" s="8">
+        <v>0</v>
+      </c>
+      <c r="AN27" s="8">
         <v>2.63</v>
       </c>
-      <c r="AN27" s="8">
-        <v>0</v>
-      </c>
       <c r="AO27" s="8">
         <v>0</v>
       </c>
@@ -5135,25 +5188,28 @@
         <v>0</v>
       </c>
       <c r="AQ27" s="8">
+        <v>0</v>
+      </c>
+      <c r="AR27" s="8">
         <v>1.76</v>
       </c>
-      <c r="AR27" s="8">
+      <c r="AS27" s="8">
         <v>0.03</v>
       </c>
-      <c r="AS27" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="AT27" s="8">
+      <c r="AT27" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="AU27" s="8">
         <v>0.28169014084506999</v>
       </c>
-      <c r="AU27" s="8">
+      <c r="AV27" s="8">
         <v>1.79</v>
       </c>
-      <c r="AV27" s="8">
+      <c r="AW27" s="8">
         <v>50.42</v>
       </c>
     </row>
-    <row r="28" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>24</v>
       </c>
@@ -5230,42 +5286,40 @@
       <c r="Z28" s="3" t="s">
         <v>361</v>
       </c>
-      <c r="AA28" s="8">
+      <c r="AA28" s="3"/>
+      <c r="AB28" s="8">
         <v>1024.77</v>
       </c>
-      <c r="AB28" s="8">
+      <c r="AC28" s="8">
         <v>689.76</v>
       </c>
-      <c r="AC28" s="8">
+      <c r="AD28" s="8">
         <v>65</v>
       </c>
-      <c r="AD28" s="3" t="s">
-        <v>375</v>
-      </c>
       <c r="AE28" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF28" s="8">
+        <v>374</v>
+      </c>
+      <c r="AF28" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AG28" s="8">
         <v>256.05</v>
       </c>
-      <c r="AG28" s="8">
+      <c r="AH28" s="8">
         <v>0.36</v>
       </c>
-      <c r="AH28" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="AI28" s="8">
+      <c r="AI28" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="AJ28" s="8">
         <v>67.308761966099993</v>
       </c>
-      <c r="AJ28" s="8">
-        <v>0</v>
-      </c>
       <c r="AK28" s="8">
+        <v>0</v>
+      </c>
+      <c r="AL28" s="8">
         <v>170.89</v>
       </c>
-      <c r="AL28" s="8">
-        <v>0</v>
-      </c>
       <c r="AM28" s="8">
         <v>0</v>
       </c>
@@ -5276,26 +5330,29 @@
         <v>0</v>
       </c>
       <c r="AP28" s="8">
+        <v>0</v>
+      </c>
+      <c r="AQ28" s="8">
         <v>518.87</v>
       </c>
-      <c r="AQ28" s="8">
+      <c r="AR28" s="8">
         <v>276.49</v>
       </c>
-      <c r="AR28" s="8">
+      <c r="AS28" s="8">
         <v>90.15</v>
       </c>
-      <c r="AS28" s="3"/>
-      <c r="AT28" s="8">
-        <v>0</v>
-      </c>
+      <c r="AT28" s="3"/>
       <c r="AU28" s="8">
+        <v>0</v>
+      </c>
+      <c r="AV28" s="8">
         <v>366.64</v>
       </c>
-      <c r="AV28" s="8">
+      <c r="AW28" s="8">
         <v>35.78</v>
       </c>
     </row>
-    <row r="29" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>25</v>
       </c>
@@ -5372,38 +5429,38 @@
         <v>154</v>
       </c>
       <c r="Z29" s="3" t="s">
-        <v>362</v>
-      </c>
-      <c r="AA29" s="8">
+        <v>416</v>
+      </c>
+      <c r="AA29" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AB29" s="8">
         <v>11</v>
       </c>
-      <c r="AB29" s="8">
+      <c r="AC29" s="8">
         <v>10.3</v>
       </c>
-      <c r="AC29" s="8">
+      <c r="AD29" s="8">
         <v>75</v>
       </c>
-      <c r="AD29" s="3" t="s">
-        <v>376</v>
-      </c>
       <c r="AE29" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF29" s="8">
-        <v>0</v>
+        <v>375</v>
+      </c>
+      <c r="AF29" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="AG29" s="8">
         <v>0</v>
       </c>
-      <c r="AH29" s="3" t="s">
+      <c r="AH29" s="8">
+        <v>0</v>
+      </c>
+      <c r="AI29" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="AI29" s="8">
+      <c r="AJ29" s="8">
         <v>93.636363636363996</v>
       </c>
-      <c r="AJ29" s="8">
-        <v>0</v>
-      </c>
       <c r="AK29" s="8">
         <v>0</v>
       </c>
@@ -5420,26 +5477,29 @@
         <v>0</v>
       </c>
       <c r="AP29" s="8">
+        <v>0</v>
+      </c>
+      <c r="AQ29" s="8">
         <v>10.3</v>
       </c>
-      <c r="AQ29" s="8">
+      <c r="AR29" s="8">
         <v>4.8</v>
       </c>
-      <c r="AR29" s="8">
+      <c r="AS29" s="8">
         <v>1.6</v>
       </c>
-      <c r="AS29" s="3"/>
-      <c r="AT29" s="8">
-        <v>0</v>
-      </c>
+      <c r="AT29" s="3"/>
       <c r="AU29" s="8">
+        <v>0</v>
+      </c>
+      <c r="AV29" s="8">
         <v>6.4</v>
       </c>
-      <c r="AV29" s="8">
+      <c r="AW29" s="8">
         <v>58.181818181818002</v>
       </c>
     </row>
-    <row r="30" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>26</v>
       </c>
@@ -5518,10 +5578,10 @@
       <c r="AB30" s="3"/>
       <c r="AC30" s="3"/>
       <c r="AD30" s="3"/>
-      <c r="AE30" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF30" s="3"/>
+      <c r="AE30" s="3"/>
+      <c r="AF30" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG30" s="3"/>
       <c r="AH30" s="3"/>
       <c r="AI30" s="3"/>
@@ -5538,8 +5598,9 @@
       <c r="AT30" s="3"/>
       <c r="AU30" s="3"/>
       <c r="AV30" s="3"/>
+      <c r="AW30" s="3"/>
     </row>
-    <row r="31" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>27</v>
       </c>
@@ -5590,10 +5651,10 @@
       <c r="AB31" s="3"/>
       <c r="AC31" s="3"/>
       <c r="AD31" s="3"/>
-      <c r="AE31" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF31" s="3"/>
+      <c r="AE31" s="3"/>
+      <c r="AF31" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
       <c r="AI31" s="3"/>
@@ -5610,8 +5671,9 @@
       <c r="AT31" s="3"/>
       <c r="AU31" s="3"/>
       <c r="AV31" s="3"/>
+      <c r="AW31" s="3"/>
     </row>
-    <row r="32" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>28</v>
       </c>
@@ -5690,10 +5752,10 @@
       <c r="AB32" s="3"/>
       <c r="AC32" s="3"/>
       <c r="AD32" s="3"/>
-      <c r="AE32" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF32" s="3"/>
+      <c r="AE32" s="3"/>
+      <c r="AF32" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
       <c r="AI32" s="3"/>
@@ -5710,8 +5772,9 @@
       <c r="AT32" s="3"/>
       <c r="AU32" s="3"/>
       <c r="AV32" s="3"/>
+      <c r="AW32" s="3"/>
     </row>
-    <row r="33" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
         <v>29</v>
       </c>
@@ -5790,15 +5853,15 @@
       <c r="AB33" s="3"/>
       <c r="AC33" s="3"/>
       <c r="AD33" s="3"/>
-      <c r="AE33" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF33" s="3"/>
+      <c r="AE33" s="3"/>
+      <c r="AF33" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG33" s="3"/>
-      <c r="AH33" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="AI33" s="3"/>
+      <c r="AH33" s="3"/>
+      <c r="AI33" s="3" t="s">
+        <v>392</v>
+      </c>
       <c r="AJ33" s="3"/>
       <c r="AK33" s="3"/>
       <c r="AL33" s="3"/>
@@ -5812,8 +5875,9 @@
       <c r="AT33" s="3"/>
       <c r="AU33" s="3"/>
       <c r="AV33" s="3"/>
+      <c r="AW33" s="3"/>
     </row>
-    <row r="34" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
         <v>30</v>
       </c>
@@ -5888,10 +5952,10 @@
       <c r="AB34" s="3"/>
       <c r="AC34" s="3"/>
       <c r="AD34" s="3"/>
-      <c r="AE34" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF34" s="3"/>
+      <c r="AE34" s="3"/>
+      <c r="AF34" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
       <c r="AI34" s="3"/>
@@ -5908,8 +5972,9 @@
       <c r="AT34" s="3"/>
       <c r="AU34" s="3"/>
       <c r="AV34" s="3"/>
+      <c r="AW34" s="3"/>
     </row>
-    <row r="35" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>31</v>
       </c>
@@ -5968,15 +6033,15 @@
       <c r="AB35" s="3"/>
       <c r="AC35" s="3"/>
       <c r="AD35" s="3"/>
-      <c r="AE35" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF35" s="3"/>
+      <c r="AE35" s="3"/>
+      <c r="AF35" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG35" s="3"/>
-      <c r="AH35" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="AI35" s="3"/>
+      <c r="AH35" s="3"/>
+      <c r="AI35" s="3" t="s">
+        <v>393</v>
+      </c>
       <c r="AJ35" s="3"/>
       <c r="AK35" s="3"/>
       <c r="AL35" s="3"/>
@@ -5990,8 +6055,9 @@
       <c r="AT35" s="3"/>
       <c r="AU35" s="3"/>
       <c r="AV35" s="3"/>
+      <c r="AW35" s="3"/>
     </row>
-    <row r="36" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
         <v>32</v>
       </c>
@@ -6052,19 +6118,19 @@
       <c r="AB36" s="3"/>
       <c r="AC36" s="3"/>
       <c r="AD36" s="3"/>
-      <c r="AE36" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF36" s="8">
-        <v>0</v>
+      <c r="AE36" s="3"/>
+      <c r="AF36" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="AG36" s="8">
         <v>0</v>
       </c>
-      <c r="AH36" s="3" t="s">
+      <c r="AH36" s="8">
+        <v>0</v>
+      </c>
+      <c r="AI36" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="AI36" s="3"/>
       <c r="AJ36" s="3"/>
       <c r="AK36" s="3"/>
       <c r="AL36" s="3"/>
@@ -6078,8 +6144,9 @@
       <c r="AT36" s="3"/>
       <c r="AU36" s="3"/>
       <c r="AV36" s="3"/>
+      <c r="AW36" s="3"/>
     </row>
-    <row r="37" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>33</v>
       </c>
@@ -6144,15 +6211,15 @@
       <c r="AB37" s="3"/>
       <c r="AC37" s="3"/>
       <c r="AD37" s="3"/>
-      <c r="AE37" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF37" s="3"/>
+      <c r="AE37" s="3"/>
+      <c r="AF37" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG37" s="3"/>
-      <c r="AH37" s="3" t="s">
+      <c r="AH37" s="3"/>
+      <c r="AI37" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="AI37" s="3"/>
       <c r="AJ37" s="3"/>
       <c r="AK37" s="3"/>
       <c r="AL37" s="3"/>
@@ -6166,8 +6233,9 @@
       <c r="AT37" s="3"/>
       <c r="AU37" s="3"/>
       <c r="AV37" s="3"/>
+      <c r="AW37" s="3"/>
     </row>
-    <row r="38" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A38" s="1" t="s">
         <v>34</v>
       </c>
@@ -6248,15 +6316,15 @@
       <c r="AB38" s="3"/>
       <c r="AC38" s="3"/>
       <c r="AD38" s="3"/>
-      <c r="AE38" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF38" s="3"/>
+      <c r="AE38" s="3"/>
+      <c r="AF38" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG38" s="3"/>
-      <c r="AH38" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="AI38" s="3"/>
+      <c r="AH38" s="3"/>
+      <c r="AI38" s="3" t="s">
+        <v>394</v>
+      </c>
       <c r="AJ38" s="3"/>
       <c r="AK38" s="3"/>
       <c r="AL38" s="3"/>
@@ -6270,8 +6338,9 @@
       <c r="AT38" s="3"/>
       <c r="AU38" s="3"/>
       <c r="AV38" s="3"/>
+      <c r="AW38" s="3"/>
     </row>
-    <row r="39" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
         <v>35</v>
       </c>
@@ -6330,10 +6399,10 @@
       <c r="AB39" s="3"/>
       <c r="AC39" s="3"/>
       <c r="AD39" s="3"/>
-      <c r="AE39" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF39" s="3"/>
+      <c r="AE39" s="3"/>
+      <c r="AF39" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
       <c r="AI39" s="3"/>
@@ -6350,8 +6419,9 @@
       <c r="AT39" s="3"/>
       <c r="AU39" s="3"/>
       <c r="AV39" s="3"/>
+      <c r="AW39" s="3"/>
     </row>
-    <row r="40" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A40" s="1" t="s">
         <v>36</v>
       </c>
@@ -6430,10 +6500,10 @@
       <c r="AB40" s="3"/>
       <c r="AC40" s="3"/>
       <c r="AD40" s="3"/>
-      <c r="AE40" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF40" s="3"/>
+      <c r="AE40" s="3"/>
+      <c r="AF40" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
       <c r="AI40" s="3"/>
@@ -6450,8 +6520,9 @@
       <c r="AT40" s="3"/>
       <c r="AU40" s="3"/>
       <c r="AV40" s="3"/>
+      <c r="AW40" s="3"/>
     </row>
-    <row r="41" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A41" s="1" t="s">
         <v>37</v>
       </c>
@@ -6514,30 +6585,30 @@
         <v>154</v>
       </c>
       <c r="Z41" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="AA41" s="8">
-        <v>0</v>
-      </c>
+        <v>362</v>
+      </c>
+      <c r="AA41" s="3"/>
       <c r="AB41" s="8">
         <v>0</v>
       </c>
       <c r="AC41" s="8">
+        <v>0</v>
+      </c>
+      <c r="AD41" s="8">
         <v>100</v>
       </c>
-      <c r="AD41" s="3" t="s">
-        <v>377</v>
-      </c>
       <c r="AE41" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF41" s="8">
-        <v>0</v>
+        <v>376</v>
+      </c>
+      <c r="AF41" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="AG41" s="8">
         <v>0</v>
       </c>
-      <c r="AH41" s="3"/>
+      <c r="AH41" s="8">
+        <v>0</v>
+      </c>
       <c r="AI41" s="3"/>
       <c r="AJ41" s="3"/>
       <c r="AK41" s="3"/>
@@ -6546,20 +6617,21 @@
       <c r="AN41" s="3"/>
       <c r="AO41" s="3"/>
       <c r="AP41" s="3"/>
-      <c r="AQ41" s="8">
-        <v>0</v>
-      </c>
+      <c r="AQ41" s="3"/>
       <c r="AR41" s="8">
         <v>0</v>
       </c>
-      <c r="AS41" s="3"/>
+      <c r="AS41" s="8">
+        <v>0</v>
+      </c>
       <c r="AT41" s="3"/>
-      <c r="AU41" s="8">
-        <v>0</v>
-      </c>
-      <c r="AV41" s="3"/>
+      <c r="AU41" s="3"/>
+      <c r="AV41" s="8">
+        <v>0</v>
+      </c>
+      <c r="AW41" s="3"/>
     </row>
-    <row r="42" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A42" s="1" t="s">
         <v>38</v>
       </c>
@@ -6618,10 +6690,10 @@
       <c r="AB42" s="3"/>
       <c r="AC42" s="3"/>
       <c r="AD42" s="3"/>
-      <c r="AE42" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF42" s="3"/>
+      <c r="AE42" s="3"/>
+      <c r="AF42" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG42" s="3"/>
       <c r="AH42" s="3"/>
       <c r="AI42" s="3"/>
@@ -6638,8 +6710,9 @@
       <c r="AT42" s="3"/>
       <c r="AU42" s="3"/>
       <c r="AV42" s="3"/>
+      <c r="AW42" s="3"/>
     </row>
-    <row r="43" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A43" s="1" t="s">
         <v>39</v>
       </c>
@@ -6718,15 +6791,15 @@
       <c r="AB43" s="3"/>
       <c r="AC43" s="3"/>
       <c r="AD43" s="3"/>
-      <c r="AE43" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF43" s="3"/>
+      <c r="AE43" s="3"/>
+      <c r="AF43" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG43" s="3"/>
-      <c r="AH43" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="AI43" s="3"/>
+      <c r="AH43" s="3"/>
+      <c r="AI43" s="3" t="s">
+        <v>395</v>
+      </c>
       <c r="AJ43" s="3"/>
       <c r="AK43" s="3"/>
       <c r="AL43" s="3"/>
@@ -6740,8 +6813,9 @@
       <c r="AT43" s="3"/>
       <c r="AU43" s="3"/>
       <c r="AV43" s="3"/>
+      <c r="AW43" s="3"/>
     </row>
-    <row r="44" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A44" s="1" t="s">
         <v>40</v>
       </c>
@@ -6814,35 +6888,33 @@
         <v>154</v>
       </c>
       <c r="Z44" s="3" t="s">
-        <v>364</v>
-      </c>
-      <c r="AA44" s="8">
+        <v>363</v>
+      </c>
+      <c r="AA44" s="3"/>
+      <c r="AB44" s="8">
         <v>0.15354899999999999</v>
       </c>
-      <c r="AB44" s="8">
+      <c r="AC44" s="8">
         <v>1.1867000000000001E-2</v>
       </c>
-      <c r="AC44" s="8">
-        <v>0</v>
-      </c>
-      <c r="AD44" s="3" t="s">
-        <v>378</v>
+      <c r="AD44" s="8">
+        <v>0</v>
       </c>
       <c r="AE44" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF44" s="3"/>
+        <v>377</v>
+      </c>
+      <c r="AF44" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
-      <c r="AI44" s="8">
+      <c r="AI44" s="3"/>
+      <c r="AJ44" s="8">
         <v>7.7284775543963002</v>
       </c>
-      <c r="AJ44" s="8">
+      <c r="AK44" s="8">
         <v>3.3916000000000002E-2</v>
       </c>
-      <c r="AK44" s="8">
-        <v>0</v>
-      </c>
       <c r="AL44" s="8">
         <v>0</v>
       </c>
@@ -6856,28 +6928,31 @@
         <v>0</v>
       </c>
       <c r="AP44" s="8">
+        <v>0</v>
+      </c>
+      <c r="AQ44" s="8">
         <v>1.1867000000000001E-2</v>
       </c>
-      <c r="AQ44" s="8">
-        <v>0</v>
-      </c>
       <c r="AR44" s="8">
+        <v>0</v>
+      </c>
+      <c r="AS44" s="8">
         <v>4.2703999999999999E-2</v>
       </c>
-      <c r="AS44" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="AT44" s="8">
+      <c r="AT44" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="AU44" s="8">
         <v>22.088063093866001</v>
       </c>
-      <c r="AU44" s="8">
+      <c r="AV44" s="8">
         <v>4.2703999999999999E-2</v>
       </c>
-      <c r="AV44" s="8">
+      <c r="AW44" s="8">
         <v>27.811317559867</v>
       </c>
     </row>
-    <row r="45" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A45" s="1" t="s">
         <v>41</v>
       </c>
@@ -6936,10 +7011,10 @@
       <c r="AB45" s="3"/>
       <c r="AC45" s="3"/>
       <c r="AD45" s="3"/>
-      <c r="AE45" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF45" s="3"/>
+      <c r="AE45" s="3"/>
+      <c r="AF45" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
       <c r="AI45" s="3"/>
@@ -6956,8 +7031,9 @@
       <c r="AT45" s="3"/>
       <c r="AU45" s="3"/>
       <c r="AV45" s="3"/>
+      <c r="AW45" s="3"/>
     </row>
-    <row r="46" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A46" s="1" t="s">
         <v>42</v>
       </c>
@@ -7036,10 +7112,10 @@
       <c r="AB46" s="3"/>
       <c r="AC46" s="3"/>
       <c r="AD46" s="3"/>
-      <c r="AE46" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF46" s="3"/>
+      <c r="AE46" s="3"/>
+      <c r="AF46" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
       <c r="AI46" s="3"/>
@@ -7056,8 +7132,9 @@
       <c r="AT46" s="3"/>
       <c r="AU46" s="3"/>
       <c r="AV46" s="3"/>
+      <c r="AW46" s="3"/>
     </row>
-    <row r="47" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A47" s="1" t="s">
         <v>43</v>
       </c>
@@ -7138,15 +7215,15 @@
       <c r="AB47" s="3"/>
       <c r="AC47" s="3"/>
       <c r="AD47" s="3"/>
-      <c r="AE47" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF47" s="3"/>
+      <c r="AE47" s="3"/>
+      <c r="AF47" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG47" s="3"/>
-      <c r="AH47" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="AI47" s="3"/>
+      <c r="AH47" s="3"/>
+      <c r="AI47" s="3" t="s">
+        <v>396</v>
+      </c>
       <c r="AJ47" s="3"/>
       <c r="AK47" s="3"/>
       <c r="AL47" s="3"/>
@@ -7160,8 +7237,9 @@
       <c r="AT47" s="3"/>
       <c r="AU47" s="3"/>
       <c r="AV47" s="3"/>
+      <c r="AW47" s="3"/>
     </row>
-    <row r="48" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A48" s="1" t="s">
         <v>44</v>
       </c>
@@ -7226,15 +7304,15 @@
       <c r="AB48" s="3"/>
       <c r="AC48" s="3"/>
       <c r="AD48" s="3"/>
-      <c r="AE48" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF48" s="3"/>
+      <c r="AE48" s="3"/>
+      <c r="AF48" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG48" s="3"/>
-      <c r="AH48" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="AI48" s="3"/>
+      <c r="AH48" s="3"/>
+      <c r="AI48" s="3" t="s">
+        <v>397</v>
+      </c>
       <c r="AJ48" s="3"/>
       <c r="AK48" s="3"/>
       <c r="AL48" s="3"/>
@@ -7248,8 +7326,9 @@
       <c r="AT48" s="3"/>
       <c r="AU48" s="3"/>
       <c r="AV48" s="3"/>
+      <c r="AW48" s="3"/>
     </row>
-    <row r="49" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A49" s="1" t="s">
         <v>45</v>
       </c>
@@ -7322,15 +7401,15 @@
       <c r="AB49" s="3"/>
       <c r="AC49" s="3"/>
       <c r="AD49" s="3"/>
-      <c r="AE49" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF49" s="3"/>
+      <c r="AE49" s="3"/>
+      <c r="AF49" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG49" s="3"/>
-      <c r="AH49" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="AI49" s="3"/>
+      <c r="AH49" s="3"/>
+      <c r="AI49" s="3" t="s">
+        <v>398</v>
+      </c>
       <c r="AJ49" s="3"/>
       <c r="AK49" s="3"/>
       <c r="AL49" s="3"/>
@@ -7344,8 +7423,9 @@
       <c r="AT49" s="3"/>
       <c r="AU49" s="3"/>
       <c r="AV49" s="3"/>
+      <c r="AW49" s="3"/>
     </row>
-    <row r="50" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A50" s="1" t="s">
         <v>46</v>
       </c>
@@ -7416,36 +7496,34 @@
         <v>154</v>
       </c>
       <c r="Z50" s="3" t="s">
-        <v>365</v>
-      </c>
-      <c r="AA50" s="8">
-        <v>0</v>
-      </c>
+        <v>364</v>
+      </c>
+      <c r="AA50" s="3"/>
       <c r="AB50" s="8">
+        <v>0</v>
+      </c>
+      <c r="AC50" s="8">
         <v>0.01</v>
       </c>
-      <c r="AC50" s="8">
+      <c r="AD50" s="8">
         <v>95</v>
       </c>
-      <c r="AD50" s="3" t="s">
-        <v>379</v>
-      </c>
       <c r="AE50" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF50" s="8">
+        <v>378</v>
+      </c>
+      <c r="AF50" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AG50" s="8">
         <v>0.03</v>
       </c>
-      <c r="AG50" s="8">
-        <v>0</v>
-      </c>
-      <c r="AH50" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="AI50" s="3"/>
-      <c r="AJ50" s="8">
-        <v>0</v>
-      </c>
+      <c r="AH50" s="8">
+        <v>0</v>
+      </c>
+      <c r="AI50" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="AJ50" s="3"/>
       <c r="AK50" s="8">
         <v>0</v>
       </c>
@@ -7453,11 +7531,11 @@
         <v>0</v>
       </c>
       <c r="AM50" s="8">
+        <v>0</v>
+      </c>
+      <c r="AN50" s="8">
         <v>0.01</v>
       </c>
-      <c r="AN50" s="8">
-        <v>0</v>
-      </c>
       <c r="AO50" s="8">
         <v>0</v>
       </c>
@@ -7470,14 +7548,17 @@
       <c r="AR50" s="8">
         <v>0</v>
       </c>
-      <c r="AS50" s="3"/>
+      <c r="AS50" s="8">
+        <v>0</v>
+      </c>
       <c r="AT50" s="3"/>
-      <c r="AU50" s="8">
-        <v>0</v>
-      </c>
-      <c r="AV50" s="3"/>
+      <c r="AU50" s="3"/>
+      <c r="AV50" s="8">
+        <v>0</v>
+      </c>
+      <c r="AW50" s="3"/>
     </row>
-    <row r="51" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A51" s="1" t="s">
         <v>47</v>
       </c>
@@ -7552,74 +7633,75 @@
         <v>154</v>
       </c>
       <c r="Z51" s="3" t="s">
-        <v>366</v>
-      </c>
-      <c r="AA51" s="8">
+        <v>365</v>
+      </c>
+      <c r="AA51" s="3"/>
+      <c r="AB51" s="8">
         <v>3.52</v>
       </c>
-      <c r="AB51" s="8">
+      <c r="AC51" s="8">
         <v>2.4300000000000002</v>
       </c>
-      <c r="AC51" s="8">
+      <c r="AD51" s="8">
         <v>85</v>
       </c>
-      <c r="AD51" s="3" t="s">
-        <v>380</v>
-      </c>
       <c r="AE51" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF51" s="8">
+        <v>379</v>
+      </c>
+      <c r="AF51" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AG51" s="8">
         <v>1.28</v>
       </c>
-      <c r="AG51" s="8">
+      <c r="AH51" s="8">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AH51" s="3"/>
-      <c r="AI51" s="8">
+      <c r="AI51" s="3"/>
+      <c r="AJ51" s="8">
         <v>69.034090909091006</v>
       </c>
-      <c r="AJ51" s="8">
+      <c r="AK51" s="8">
         <v>1.1100000000000001</v>
       </c>
-      <c r="AK51" s="8">
-        <v>0</v>
-      </c>
       <c r="AL51" s="8">
         <v>0</v>
       </c>
       <c r="AM51" s="8">
+        <v>0</v>
+      </c>
+      <c r="AN51" s="8">
         <v>2.2000000000000002</v>
       </c>
-      <c r="AN51" s="8">
-        <v>0</v>
-      </c>
       <c r="AO51" s="8">
+        <v>0</v>
+      </c>
+      <c r="AP51" s="8">
         <v>0.23</v>
       </c>
-      <c r="AP51" s="8">
-        <v>0</v>
-      </c>
       <c r="AQ51" s="8">
+        <v>0</v>
+      </c>
+      <c r="AR51" s="8">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="AR51" s="8">
+      <c r="AS51" s="8">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="AS51" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="AT51" s="8">
+      <c r="AT51" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="AU51" s="8">
         <v>31.534090909090999</v>
       </c>
-      <c r="AU51" s="8">
+      <c r="AV51" s="8">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="AV51" s="8">
+      <c r="AW51" s="8">
         <v>1.4772727272727</v>
       </c>
     </row>
-    <row r="52" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A52" s="1" t="s">
         <v>48</v>
       </c>
@@ -7698,10 +7780,10 @@
       <c r="AB52" s="3"/>
       <c r="AC52" s="3"/>
       <c r="AD52" s="3"/>
-      <c r="AE52" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF52" s="3"/>
+      <c r="AE52" s="3"/>
+      <c r="AF52" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
       <c r="AI52" s="3"/>
@@ -7718,8 +7800,9 @@
       <c r="AT52" s="3"/>
       <c r="AU52" s="3"/>
       <c r="AV52" s="3"/>
+      <c r="AW52" s="3"/>
     </row>
-    <row r="53" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A53" s="1" t="s">
         <v>49</v>
       </c>
@@ -7794,15 +7877,15 @@
       <c r="AB53" s="3"/>
       <c r="AC53" s="3"/>
       <c r="AD53" s="3"/>
-      <c r="AE53" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF53" s="3"/>
+      <c r="AE53" s="3"/>
+      <c r="AF53" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG53" s="3"/>
-      <c r="AH53" s="3" t="s">
-        <v>401</v>
-      </c>
-      <c r="AI53" s="3"/>
+      <c r="AH53" s="3"/>
+      <c r="AI53" s="3" t="s">
+        <v>400</v>
+      </c>
       <c r="AJ53" s="3"/>
       <c r="AK53" s="3"/>
       <c r="AL53" s="3"/>
@@ -7816,8 +7899,9 @@
       <c r="AT53" s="3"/>
       <c r="AU53" s="3"/>
       <c r="AV53" s="3"/>
+      <c r="AW53" s="3"/>
     </row>
-    <row r="54" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A54" s="1" t="s">
         <v>50</v>
       </c>
@@ -7896,10 +7980,10 @@
       <c r="AB54" s="3"/>
       <c r="AC54" s="3"/>
       <c r="AD54" s="3"/>
-      <c r="AE54" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF54" s="3"/>
+      <c r="AE54" s="3"/>
+      <c r="AF54" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
       <c r="AI54" s="3"/>
@@ -7916,8 +8000,9 @@
       <c r="AT54" s="3"/>
       <c r="AU54" s="3"/>
       <c r="AV54" s="3"/>
+      <c r="AW54" s="3"/>
     </row>
-    <row r="55" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A55" s="1" t="s">
         <v>51</v>
       </c>
@@ -7994,15 +8079,15 @@
       <c r="AB55" s="3"/>
       <c r="AC55" s="3"/>
       <c r="AD55" s="3"/>
-      <c r="AE55" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="AF55" s="3"/>
+      <c r="AE55" s="3"/>
+      <c r="AF55" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="AG55" s="3"/>
-      <c r="AH55" s="3" t="s">
-        <v>402</v>
-      </c>
-      <c r="AI55" s="3"/>
+      <c r="AH55" s="3"/>
+      <c r="AI55" s="3" t="s">
+        <v>401</v>
+      </c>
       <c r="AJ55" s="3"/>
       <c r="AK55" s="3"/>
       <c r="AL55" s="3"/>
@@ -8016,8 +8101,9 @@
       <c r="AT55" s="3"/>
       <c r="AU55" s="3"/>
       <c r="AV55" s="3"/>
+      <c r="AW55" s="3"/>
     </row>
-    <row r="56" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A56" s="1" t="s">
         <v>52</v>
       </c>
@@ -8094,90 +8180,85 @@
         <v>154</v>
       </c>
       <c r="Z56" s="3" t="s">
-        <v>367</v>
-      </c>
-      <c r="AA56" s="8">
+        <v>366</v>
+      </c>
+      <c r="AA56" s="3"/>
+      <c r="AB56" s="8">
         <v>153.41999999999999</v>
       </c>
-      <c r="AB56" s="8">
+      <c r="AC56" s="8">
         <v>179.27344751000001</v>
       </c>
-      <c r="AC56" s="8">
+      <c r="AD56" s="8">
         <v>80</v>
       </c>
-      <c r="AD56" s="3" t="s">
-        <v>381</v>
-      </c>
       <c r="AE56" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF56" s="8">
+        <v>380</v>
+      </c>
+      <c r="AF56" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="AG56" s="8">
         <v>43.12</v>
       </c>
-      <c r="AG56" s="8">
+      <c r="AH56" s="8">
         <v>0.01</v>
       </c>
-      <c r="AH56" s="3" t="s">
-        <v>403</v>
-      </c>
-      <c r="AI56" s="8">
+      <c r="AI56" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="AJ56" s="8">
         <v>116.85141931299999</v>
       </c>
-      <c r="AJ56" s="8">
+      <c r="AK56" s="8">
         <v>3.92</v>
       </c>
-      <c r="AK56" s="8">
-        <v>0</v>
-      </c>
       <c r="AL56" s="8">
         <v>0</v>
       </c>
       <c r="AM56" s="8">
+        <v>0</v>
+      </c>
+      <c r="AN56" s="8">
         <v>67.03728606</v>
       </c>
-      <c r="AN56" s="8">
-        <v>0</v>
-      </c>
       <c r="AO56" s="8">
+        <v>0</v>
+      </c>
+      <c r="AP56" s="8">
         <v>0.13652955</v>
       </c>
-      <c r="AP56" s="8">
+      <c r="AQ56" s="8">
         <v>112.09963190000001</v>
       </c>
-      <c r="AQ56" s="8">
+      <c r="AR56" s="8">
         <v>26.377127389999998</v>
       </c>
-      <c r="AR56" s="8">
+      <c r="AS56" s="8">
         <v>14.717837960000001</v>
       </c>
-      <c r="AS56" s="3" t="s">
-        <v>411</v>
-      </c>
-      <c r="AT56" s="8">
+      <c r="AT56" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="AU56" s="8">
         <v>2.5550775648545998</v>
       </c>
-      <c r="AU56" s="8">
+      <c r="AV56" s="8">
         <v>41.094965350000003</v>
       </c>
-      <c r="AV56" s="8">
+      <c r="AW56" s="8">
         <v>26.79</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:AV56" xr:uid="{22618D3F-C01D-44CF-9330-E09D0B7E4ED3}"/>
+  <autoFilter ref="A3:AW56" xr:uid="{22618D3F-C01D-44CF-9330-E09D0B7E4ED3}"/>
   <mergeCells count="5">
-    <mergeCell ref="AI1:AV1"/>
+    <mergeCell ref="AJ1:AW1"/>
     <mergeCell ref="E1:K1"/>
     <mergeCell ref="M1:X1"/>
-    <mergeCell ref="Y1:AD1"/>
-    <mergeCell ref="AE1:AH1"/>
+    <mergeCell ref="Y1:AE1"/>
+    <mergeCell ref="AF1:AI1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{3de9faa6-9fe1-49b3-9a08-227a296b54a6}" enabled="1" method="Privileged" siteId="{66d73691-ea97-48b1-95d5-e94f0a46b878}" contentBits="0" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>